<commit_message>
Adding Kiswahili translation to household registration form
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56" count="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="60" count="60">
   <si>
     <t>type</t>
   </si>
@@ -111,6 +111,9 @@
     <t>kitongoji</t>
   </si>
   <si>
+    <t>Kitongoji:</t>
+  </si>
+  <si>
     <t>house_number</t>
   </si>
   <si>
@@ -165,6 +168,9 @@
     <t>Use one of the following formats: +255XXXXXXXXX or 0XXXXXXXXX.</t>
   </si>
   <si>
+    <t>Tumia moja kati ya mfumo huu +255XXXXXXXXX au 0XXXXXXXXX.</t>
+  </si>
+  <si>
     <t>repeat</t>
   </si>
   <si>
@@ -186,10 +192,16 @@
     <t>Yes</t>
   </si>
   <si>
+    <t>Ndiyo</t>
+  </si>
+  <si>
     <t>no</t>
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Hapana</t>
   </si>
   <si>
     <t>yes_no_think</t>
@@ -297,7 +309,7 @@
     <col min="11" max="11" style="0" width="23.141466346153848" bestFit="1" customWidth="1"/>
     <col min="12" max="12" style="0" width="56.282331730769236" customWidth="1"/>
     <col min="13" max="13" style="0" width="31.426682692307697" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" style="0" width="354.97866586538464" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" style="0" width="28.56971153846154" customWidth="1"/>
     <col min="15" max="16" style="0" width="7.9995192307692315" bestFit="1" customWidth="1"/>
     <col min="17" max="17" style="0" width="23.284314903846155" bestFit="1" customWidth="1"/>
     <col min="18" max="16384" style="0" width="9.142307692307693"/>
@@ -753,6 +765,11 @@
           <t>Household Location</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Eneo la kaya</t>
+        </is>
+      </c>
       <c r="G27" t="s">
         <v>14</v>
       </c>
@@ -771,6 +788,11 @@
           <t>_The purpose of the following questions regarding the household location is to help you locate this house again when it is time to return for another visit to the people who live here. Enter the information that you will need to help you easily find this house again when you need to before you approach the household. What is the address of this household?_</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hiyi pindi unapotaka kuirudia tena. Kabla ya kuifika kaya hii. Ni ipi anuani ya nyumba hii?</t>
+        </is>
+      </c>
       <c r="G28" t="s">
         <v>14</v>
       </c>
@@ -782,10 +804,11 @@
       <c r="B29" t="s">
         <v>27</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Kitongoji:</t>
-        </is>
+      <c r="C29" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" t="s">
+        <v>28</v>
       </c>
       <c r="E29" t="s">
         <v>19</v>
@@ -796,11 +819,16 @@
         <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
           <t>House number:</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Nambari ya nyumba</t>
         </is>
       </c>
       <c r="E30" t="s">
@@ -811,17 +839,27 @@
           <t>Enter the entire house number separated by slashes</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Ingiza nambari ya nyumba yote na tenganisha kwa kutumia alama ya Mkwaju</t>
+        </is>
+      </c>
     </row>
     <row r="31" spans="1:17" customHeight="1" ht="13.5">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>How many minutes does it take you to travel between this home and your home?</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Ni dakika ngapi unatumia kutoka nyumbani kwenu hadi kwenye nyumba hii?</t>
         </is>
       </c>
       <c r="E31" t="s">
@@ -842,6 +880,11 @@
       <c r="C32" t="inlineStr">
         <is>
           <t>How do you travel between your home and this home?</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Unatumia usafiri gani?</t>
         </is>
       </c>
       <c r="E32" t="s">
@@ -853,11 +896,16 @@
         <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
           <t>Specify other means of travel:</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Taja aina nyengine ya usafiri</t>
         </is>
       </c>
       <c r="E33" t="s">
@@ -865,7 +913,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>selected(${means_of_travel},"other")</t>
+          <t>selected(${means_of_travel_house},"other")</t>
         </is>
       </c>
     </row>
@@ -883,6 +931,11 @@
       <c r="N34" t="inlineStr">
         <is>
           <t>Make sure location services on your phone are turned on.</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Hakikisha unawasha GPS kwenye simu yako</t>
         </is>
       </c>
     </row>
@@ -899,12 +952,12 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:17" customHeight="1" ht="13.5">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -915,6 +968,12 @@
         <is>
           <t>Now, approach the household. Introduce yourself and ask how many families (kayas) are living in this house. If more than one, ask if all heads of families are available and ready to speak at this time (Mhusi ka mkuu wa hii nyumba yupo?). If one head of family is away or not available to speak, or the heads of the families are not ready to be on the same conversation, speak with each family separately.  
 Is at least one head of family available to speak at this time?</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Nenda kwenye nyumba, jitambulishe na uliza je kwenye nyumba hii munaishi (kaya) ngapi?  Ikiwa muna kaya zaidi ya moja uliza je wakuu wa kaya wapo na tunaweza kuzungumza mda huu?  Ikiwa mkuu wa kaya mmoja hayupo au hayuko tayari kuzungumza au hayupo huru kujichanganya kwenye mazungumzo pamoja na mwenziwe, jaribu kuzungumza na mkuu wa kaya mmoja halafu zungumza na mwengine.
+Je yupo mkuu wa kaya japo mmoja  kwenye nyumba hii aliye tayari kuzungumza?</t>
         </is>
       </c>
       <c r="E37" t="s">
@@ -935,12 +994,22 @@
           <t>Since the head of the family is not available to speak to you now, you can move on to the next household. Come back to the house in a few days and try to register the family again.</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Ikiwa mkuu wa kaya hayupo au hawezi kuzungumza na wewe saahivi. Unaweza kwenda nyumba nyengine. Tutakuekea alama ya kukukumbusha kurudi tena kwenye nyumba hii siku chache baadae ili kumaliza usajili.</t>
+        </is>
+      </c>
       <c r="F38" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
           <t>You should now exit this form.</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Sasa toka kwenye fomu hii.</t>
         </is>
       </c>
     </row>
@@ -954,7 +1023,7 @@
         </is>
       </c>
       <c r="F39" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -967,7 +1036,7 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:17" customHeight="1" ht="13.5">
@@ -975,7 +1044,7 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1002,10 +1071,21 @@
 _Allow the family to ask any questions they may have_</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Jitambulishe wewe ni nani, na jukumu lako kama muhudumu wa afya  wa kujitolea wa jamii, mambo muhimu ya kuzingatia ni haya:
+Hizi ni jitihada za kitaifa zilizowekwa na Wizara ya Afya ili kuboresha huduma za afya kwa jamii Zanzibar. Kila eneo saahivi litakuwa na muhudumu wa afya wa kujitoea wa jamii, ambaye atashughulika na wamama wajawazito, watoto walio na umri chini ya miaka 5 na mambo yote ya kiafya yanayowahusu watoto, lishe na maendeleo ya mtoto.
+Mwanzoni nitaisajili kaya yako na kukuuliza maswali ya msingi yatayoniwezesha kujua ni watu wangapi wanaoishi katika eneo langu na mahitaji yao ya kiafya. Kila atapojitokeza mteja mpya katika kaya nitawaomba ridhaa au ridhaa ya wazee niwasajili na niwatembelee ili kuwapatia huduma za afya. Kwasasa nitajikita kuwasaidia wamama wajawazito kuwa na afya bora na kuhakikisha kuwa anajifungua salama na mtoto anayezaliwa na watoto wengine wanakuwa katika hali imara na afya bora.  Mbeleni huenda nikawasaidia watu wengine kwenye kaya hii kuishi maisha ya afya bora zaidi.
+Baadhi ya majukumu yangu kama muhumu wa afya wa kuitolea ni kutoa elimu ya afya, kuchunguza dalili za hatari, kutoa rufaa pale itapohitajika na kuzifuatilia, nitahakikisha familia yako inapata taarifa zote za afya inazozihitahi kwa muda stahili. Asante sana.
+Kwasasababu mimi si daktari, wala nesi nitatumia simu yangu hii ya kisasa kufanya matembeleo, simu hii ina muongozo ambao utanisaidia kufanya kazi yangu kwa ufanisi na kueka  kumbukumbu ya matembelo yangu. Naomba niwahakikishie kuwa mazungumzo yetu yatabaki kuwa siri na hayatatolewa kwa mtu yeyote au popopte.
+Pia ningependa kukueleza kwanini ni muhimu kwa familia yako kusajiliwa katika mradi huu. Ushiriki wako katika mradi huu wa kitaifa wa afya utaisaidia serekali kukuza utowaji wahuduma za afya Nchini. Pia itakupa nafasi ya kujifunza mahitaji ya afya ya familia yako hasa katika maswala yanayohusu ujauzito/huduma stahiki za mama na mtoto baada ya kujifungua na kuwawezesha kupata huduma za afya wanazohitaji ili kuboresha ustawi wa familia yako.
+_Iruhusu familia ikuulize maswali yoyote waliyonayo_</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="1:17" customHeight="1" ht="13.5">
       <c r="A43" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1015,6 +1095,11 @@
       <c r="C43" t="inlineStr">
         <is>
           <t>ENTER: Is there more than one kaya living in this house?</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>INGIA: Je kuna kaya zaidi ya moja inayoishi humu?</t>
         </is>
       </c>
       <c r="E43" t="s">
@@ -1036,8 +1121,14 @@
 SAY: At this point I'd like to speak to each of you individually about getting some more information about the members of your family.</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Anza kusajili kaya moja kwenda nyengine. Jikite mazungumzo yako kwa mkuu wa kaya wa kwanza omba ridhaa yake kuwasajili wanafamiliwa wake. Ukimaliza kaya ya kwanza, Anza usajili kwa mkuu wa kaya mwengine.
+SEMA: Saahizi ningependa nizungumze na nyinyi mmoja mmoja ili nipate taarifa zaidi kuhusu wanafamilia wenu.</t>
+        </is>
+      </c>
       <c r="F44" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45" spans="1:17" customHeight="1" ht="13.5">
@@ -1054,6 +1145,11 @@
           <t>Continue with the registration process for the people in this kaya.</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Endelea na mchakato wa usajili kwa watu waliomo kwenye kaya hii.</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>selected(${other_kayas},"no")</t>
@@ -1074,6 +1170,11 @@
       <c r="C46" t="inlineStr">
         <is>
           <t>ASK: Are you willing to register your household?</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ULIZA: Je uko tayari kusajili kaya yako?</t>
         </is>
       </c>
       <c r="E46" t="s">
@@ -1085,7 +1186,7 @@
         <v>4</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1095,7 +1196,7 @@
     </row>
     <row r="48" spans="1:17" customHeight="1" ht="13.5">
       <c r="A48" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1105,6 +1206,11 @@
       <c r="C48" t="inlineStr">
         <is>
           <t>SAY: I understand that you are not ready to register your family at this time. Could I return in a few days to discuss the services I can provide further?</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SEMA: naelewa huko tayari kuisajili kaya yako muda huu. Je naweza kurudi tena siku chache mbeleni ili tuje tujadili zaidi kuhusu huduma ambazo nitazitoa?</t>
         </is>
       </c>
       <c r="E48" t="s">
@@ -1125,6 +1231,11 @@
           <t>Thank the family for their time, and provide your contact information. Let them know that they're free to reach out at any time if they have questions about their health.</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Washukuru familia kwa kutumia muda wao na wape namba zako za simu. Waambie kuwa wako huru kukupigia muda wowote wakiwa na suali lolote kuhusu afya zao.</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>selected(${permission_to_return},"no")</t>
@@ -1132,7 +1243,12 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Your application will not schedule any more visits to this family at this time. If they become interested at a later date you can always start providing services to them. If there are any other kayas living in this house, start a new household registration process and ask the other head of the family for permission to register the members of his family.  Now you should exit this form.</t>
+          <t>Your application will not schedule any more visits to this family at this time. If they become interested at a later date you can always start providing services to them. If there are any other kayas living in this house, start a new household registration process and ask the other head of the family for permission to register the members of his family.  You should now exit this form.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Programu yako haitapanga ratiba nyengine yoyote ya familia hii kwa wakati huu. Ikiwa watahamasika baadae unaweza kuwapatia huduma. Ikiwa kuna kaya yoyote inayoihsi kwenye nyumba hii, anza mchakato mpya wa usajili na muombe ridhaa mkuu wa kaya ili kuwasajili wanakaya wake.  Sasa toka kwenye fomu hii.</t>
         </is>
       </c>
     </row>
@@ -1150,6 +1266,11 @@
           <t>SAY: OK, I understand that you're not interested right now. I'll return in a few days to discuss this further.</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>SEMA: OK naelewa kwa saivi hamukuhamasika. Nitarejea siku chache mbeleni tuzidi kujadiliana.</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>selected(${permission_to_return},"yes")</t>
@@ -1158,6 +1279,11 @@
       <c r="N50" t="inlineStr">
         <is>
           <t>Return to the household in a few days to further discuss registering the family. If there are any other kayas living in this house, start a new household registration process and ask the other head of the family for permission to register the members of his family.  Now you should exit this form</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Rejea kwenye Nyumba baada ya siku chache ili kujadili zaidi kuhusu suala la kuisajili kaya. Ikiwa kuna kaya nyengine zinazoishi kwenye nyumba hii, Anza upya mchakato wa kuisajili omba ridhaa kutoka kwa mkuu wa kaya ili uisajili kaya yake. Sasa toka kwenye fomu hii.</t>
         </is>
       </c>
     </row>
@@ -1175,8 +1301,13 @@
           <t>Once you've finished the conversation with the head of this kaya, remember to re-start a new household registration process for the other kaya(s) living in this house if you have not done so already.</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pindi ukimaliza mazungumzo na mkuu wa kaya hii, kumbuka kuirudia kaya nyengine inayoishi kwenye nyumba hii ili kufanya mchakato wa kuisajili ikiwa bado hujaisajili.</t>
+        </is>
+      </c>
       <c r="F51" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52" spans="1:17" customHeight="1" ht="13.5">
@@ -1184,7 +1315,7 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="53" spans="1:17" customHeight="1" ht="13.5">
@@ -1192,7 +1323,7 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="54" spans="1:17" customHeight="1" ht="13.5">
@@ -1200,15 +1331,15 @@
         <v>4</v>
       </c>
       <c r="B54" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="55" spans="1:17" customHeight="1" ht="13.5">
       <c r="A55" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1218,6 +1349,11 @@
       <c r="C55" t="inlineStr">
         <is>
           <t>ASK: How many people live in your Kaya?</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni watu wangapi wanaishi kwenye kaya yako?</t>
         </is>
       </c>
       <c r="E55" t="s">
@@ -1226,6 +1362,11 @@
       <c r="N55" t="inlineStr">
         <is>
           <t>Ask the person to list the names of all people who live in the house, and count to ensure that the number they provided is correct. Long term visitors to the house, such as a woman returning home for delivery, should not be counted â only people who are permanent residents of the house.</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Muombe mwenyeji wako aorodheshe majina ya watu wanaoishi kwenye kaya, na hesabu ili kuhakikisha idadi ni sawa. Usiwahesabu wageni walikokuja kutembea kwa muda mrefu, mfano wanawake walikuja nyumbani ili kujifungua, hesabu wakaazi wakudumu peke yao.</t>
         </is>
       </c>
     </row>
@@ -1243,13 +1384,18 @@
           <t>SAY: For each person, I will ask some basic details about who they are, starting with the primary contact person for this household. Who should I list as the primary contact for this household, who will be the person I reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu , tukianza na mtu ambaye naweza kuwasiliana naye kwenye nyumba hii,. Je ni nani nimuorodheshe kama mtu wa kuwasiliana naye kwenye kaya hii, Je ni nani atakayekuwa mtu ninayeweza kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia. Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
+        </is>
+      </c>
     </row>
     <row r="57" spans="1:17" customHeight="1" ht="13.5">
       <c r="A57" t="s">
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:17" customHeight="1" ht="13.5">
@@ -1257,15 +1403,20 @@
         <v>4</v>
       </c>
       <c r="B58" t="s">
+        <v>41</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Household Contact Information</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tarifa za mawasiliano za kaya</t>
+        </is>
+      </c>
+      <c r="F58" t="s">
         <v>40</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Household Contact Information</t>
-        </is>
-      </c>
-      <c r="F58" t="s">
-        <v>39</v>
       </c>
       <c r="G58" t="s">
         <v>14</v>
@@ -1285,6 +1436,11 @@
           <t>ASK: What is the first name of the best contact person for your household?</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ULIZA: ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
+        </is>
+      </c>
       <c r="E59" t="s">
         <v>19</v>
       </c>
@@ -1299,7 +1455,12 @@
         </is>
       </c>
       <c r="C60" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ULIZA: ni lipi jina la babu yake?</t>
+        </is>
       </c>
       <c r="E60" t="s">
         <v>19</v>
@@ -1322,7 +1483,7 @@
     </row>
     <row r="62" spans="1:17" customHeight="1" ht="13.5">
       <c r="A62" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1332,6 +1493,11 @@
       <c r="C62" t="inlineStr">
         <is>
           <t>Enter ${first_name_contact}'s sex:</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Ingiza jinsia yake </t>
         </is>
       </c>
       <c r="E62" t="s">
@@ -1340,7 +1506,7 @@
     </row>
     <row r="63" spans="1:17" customHeight="1" ht="13.5">
       <c r="A63" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1350,6 +1516,11 @@
       <c r="C63" t="inlineStr">
         <is>
           <t>ASK: Do you know ${first_name_contact}'s exact date of birth?</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ULIZA: Je unaijua tarehe sahihi yake ya  kuzaliwa</t>
         </is>
       </c>
       <c r="E63" t="s">
@@ -1358,7 +1529,7 @@
     </row>
     <row r="64" spans="1:17" customHeight="1" ht="13.5">
       <c r="A64" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1368,6 +1539,11 @@
       <c r="C64" t="inlineStr">
         <is>
           <t>ASK: In what year was ${first_name_contact} born?</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ULIZA Ni mwaka gani alizaliwa?</t>
         </is>
       </c>
       <c r="E64" t="s">
@@ -1388,10 +1564,15 @@
           <t>Age must be between 12 and 100!</t>
         </is>
       </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Umri uwe ni kati ya 12 na 100</t>
+        </is>
+      </c>
     </row>
     <row r="65" spans="1:17" customHeight="1" ht="13.5">
       <c r="A65" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1401,6 +1582,11 @@
       <c r="C65" t="inlineStr">
         <is>
           <t>ASK: What is ${first_name_contact}'s date of birth?</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ULIZA: Je ni ipi tarehe yake kuzaliwa?</t>
         </is>
       </c>
       <c r="E65" t="s">
@@ -1419,6 +1605,11 @@
       <c r="J65" t="inlineStr">
         <is>
           <t>Calculated age must be between 12 and 100!</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Umri uliohesabiwa ni lazima uwe kati ya miaka 12 na 100</t>
         </is>
       </c>
     </row>
@@ -1436,14 +1627,22 @@
           <t>ASK: What is the best contact phone number for ${first_name_contact}?</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ULIZA: Je ni ipi nambari yake nzuri ya mawasilaano.</t>
+        </is>
+      </c>
       <c r="E66" t="s">
         <v>19</v>
       </c>
       <c r="I66" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J66" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="K66" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="67" spans="1:17" customHeight="1" ht="13.5">
@@ -1460,15 +1659,28 @@
           <t>ASK: is there another phone number used by ${first_name_contact} or another member of the household?</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ULIZA: Je kuna nambari ya ziada anayotumia kuwasilaina?</t>
+        </is>
+      </c>
       <c r="I67" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J67" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="K67" t="s">
+        <v>47</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
           <t>You can leave this blank if there is only one good contact number for this household</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Unaweza acha pengo usijijaze chochote kama kuna nambari moja tu ya mawasiliano kwenye kaya hii</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1734,7 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="72" spans="1:17" customHeight="1" ht="13.5">
@@ -1530,7 +1742,7 @@
         <v>4</v>
       </c>
       <c r="B72" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -1545,15 +1757,20 @@
         </is>
       </c>
       <c r="B73" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
           <t>Household Member Information</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Taarifa za wanakaya</t>
+        </is>
+      </c>
       <c r="F73" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G73" t="s">
         <v>14</v>
@@ -1578,6 +1795,11 @@
           <t>Now, please enter information for the other members of the kaya.</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Sasa, tafadhali ingiza taarifa za watu wengine wanaishin kwenye kaya. </t>
+        </is>
+      </c>
     </row>
     <row r="75" spans="1:17" customHeight="1" ht="13.5">
       <c r="A75" t="s">
@@ -1624,6 +1846,11 @@
           <t>ASK: What is their first name?</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni lipi jina lake la kwanza</t>
+        </is>
+      </c>
       <c r="E77" t="s">
         <v>19</v>
       </c>
@@ -1636,7 +1863,12 @@
         <v>20</v>
       </c>
       <c r="C78" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni lipi jina lake la Babu</t>
+        </is>
       </c>
       <c r="E78" t="s">
         <v>19</v>
@@ -1687,7 +1919,7 @@
     </row>
     <row r="82" spans="1:17" customHeight="1" ht="13.5">
       <c r="A82" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B82" t="s">
         <v>21</v>
@@ -1697,6 +1929,11 @@
           <t>Enter ${first_name_c}'s sex</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Ingiza jinsia yake</t>
+        </is>
+      </c>
       <c r="E82" t="s">
         <v>19</v>
       </c>
@@ -1718,7 +1955,7 @@
     </row>
     <row r="84" spans="1:17" customHeight="1" ht="13.5">
       <c r="A84" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
@@ -1728,6 +1965,11 @@
           <t>ASK: Do you know ${first_name_c}'s exact date of birth?</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ULIZA: Je unaituja terehe yake ya kuzaliwa kwa usahihi?</t>
+        </is>
+      </c>
       <c r="E84" t="s">
         <v>19</v>
       </c>
@@ -1749,7 +1991,7 @@
     </row>
     <row r="86" spans="1:17" customHeight="1" ht="13.5">
       <c r="A86" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -1759,6 +2001,11 @@
       <c r="C86" t="inlineStr">
         <is>
           <t>ASK: Is ${first_name_c} under 5 years old?</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ULIZA: Je mtoto yupo chini yaumri wa miaka 5?</t>
         </is>
       </c>
       <c r="E86" t="s">
@@ -1784,6 +2031,11 @@
           <t>SAY: For children under 5, I'd like to try and get some more specific information about their age. Can you try and remember the year and month when ${first_name_c} was born?</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>SEMA: Kwa watoto walio chini ya miaka 5 ningependa kupata taarifa zaid kuhusu umri wao, je unaweza kukumbuka ni mwezi na mwaka gani mtoto huyu alizaliwa?</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes")</t>
@@ -1792,12 +2044,17 @@
       <c r="N87" t="inlineStr">
         <is>
           <t>It's important to try and get more exact age information for children. You can enter the child's date of birth as the first of the month in which they were born.</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Ni muhimu kupata taarifa za uhakika kuhuru umri wa watoto. Unaweza kuingiza tarehe ya mwezi wa mtoto aliozaliwa </t>
         </is>
       </c>
     </row>
     <row r="88" spans="1:17" customHeight="1" ht="13.5">
       <c r="A88" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -1807,6 +2064,11 @@
       <c r="C88" t="inlineStr">
         <is>
           <t>ASK: In what year was ${first_name_c} born?</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni mwaka gani alizaliwa?</t>
         </is>
       </c>
       <c r="E88" t="s">
@@ -1827,10 +2089,15 @@
           <t>For children under 5 years of age, a more exact birthdate must be captured.</t>
         </is>
       </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
+        </is>
+      </c>
     </row>
     <row r="89" spans="1:17" customHeight="1" ht="13.5">
       <c r="A89" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -1840,6 +2107,11 @@
       <c r="C89" t="inlineStr">
         <is>
           <t>ASK: What is ${first_name_c}'s date of birth?</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ULIZA: Ipi ni tarehe yake kuzaliwa</t>
         </is>
       </c>
       <c r="E89" t="s">
@@ -1858,6 +2130,11 @@
       <c r="J89" t="inlineStr">
         <is>
           <t>You've entered an invalid age - confirm that you've entered it properly.  For children under 5, confirm that the date is not more than 5 years ago.</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
         </is>
       </c>
     </row>
@@ -1933,6 +2210,11 @@
           <t>SAY: From this registration, I've seen that you have a child under 5 who can benefit from this national program. Therefore, I'm asking for your permission to come back and check up on all issues related to their health care, nutrition, and child development. I would be grateful for your permission.</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>SEMA kutokanana usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe na maendeleo yao.nitafurahi kama nitapata ridhaa yenu. </t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>${is_under_5_binary}=1</t>
@@ -1953,6 +2235,11 @@
           <t>SAY: I see that there are some women of reproductive age in your family. I'd like to ask your permission to return later to speak with them personally about issues related to health during pregnancy and childbirth.</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>SEMA: Nimeona kuna baadhi ya wanawake walio katika umri wa uzazi katika kaya yako. Ningeomba ridhaa yako kurudia ili kuja kuzungumza nao mambo muhimu ya afya kipindi cha ujauzito na baada ya kujifungua.</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>${reproductive_age} = 1 or ${reproductive_age_c} = 1  </t>
@@ -1987,7 +2274,7 @@
         </is>
       </c>
       <c r="B97" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:17" customHeight="1" ht="13.5">
@@ -1995,7 +2282,7 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="99" spans="1:17" customHeight="1" ht="13.5">
@@ -2012,16 +2299,21 @@
           <t>_The registration process for this kaya is now complete._</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>_Mchakato wa usajili katika kaya umekamilika_</t>
+        </is>
+      </c>
     </row>
     <row r="100" spans="1:17" customHeight="1" ht="13.5">
       <c r="A100" t="s">
         <v>4</v>
       </c>
       <c r="B100" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F100" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="101" spans="1:17" customHeight="1" ht="13.5">
@@ -2032,7 +2324,7 @@
         <v>15</v>
       </c>
       <c r="C101" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L101" t="s">
         <v>16</v>
@@ -2049,7 +2341,7 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L102" t="inlineStr">
         <is>
@@ -2085,7 +2377,7 @@
         <v>13</v>
       </c>
       <c r="C104" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
@@ -2156,7 +2448,7 @@
         <v>11</v>
       </c>
       <c r="B108" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -2174,7 +2466,7 @@
         <v>11</v>
       </c>
       <c r="B109" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -2192,7 +2484,7 @@
         <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -2210,7 +2502,7 @@
         <v>11</v>
       </c>
       <c r="B111" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -2248,7 +2540,7 @@
         <v>10</v>
       </c>
       <c r="B113" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2296,63 +2588,63 @@
     </row>
     <row r="2" spans="1:4" ht="14.25">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Ndiyo</t>
-        </is>
+        <v>54</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.25">
       <c r="A3" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Hapana</t>
-        </is>
+        <v>57</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.25">
       <c r="A4" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="D4" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="14.25">
       <c r="A5" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D5" s="2"/>
+        <v>57</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="14.25">
       <c r="A6" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -2364,7 +2656,11 @@
           <t>I need more time to decide</t>
         </is>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nahitaji muda zaidi ili kufanya maamuzi</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:4" ht="14.25">
       <c r="A7" s="2" t="s">
@@ -2380,7 +2676,11 @@
           <t>Male</t>
         </is>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Mwanamme</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:4" ht="14.25">
       <c r="A8" s="2" t="s">
@@ -2396,11 +2696,15 @@
           <t>Female</t>
         </is>
       </c>
-      <c r="D8" s="2"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Mwanamke</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:4" ht="14.25">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -2412,11 +2716,15 @@
           <t>Walk</t>
         </is>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kutembea</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="1:4" ht="14.25">
       <c r="A10" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -2428,11 +2736,15 @@
           <t>Bicycle</t>
         </is>
       </c>
-      <c r="D10" s="2"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Baskeli</t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:4" ht="14.25">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -2444,11 +2756,15 @@
           <t>Moto</t>
         </is>
       </c>
-      <c r="D11" s="2"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pikipiki/vespa au vyombo vya maringi mawili vinavyotumia mafuta</t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="14.25">
       <c r="A12" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -2460,11 +2776,15 @@
           <t>Private car</t>
         </is>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Gari binafsi</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:4" ht="14.25">
       <c r="A13" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -2476,11 +2796,15 @@
           <t>Public bus</t>
         </is>
       </c>
-      <c r="D13" s="2"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Gari ya abiria</t>
+        </is>
+      </c>
     </row>
     <row r="14" spans="1:4" ht="14.25">
       <c r="A14" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -2492,11 +2816,15 @@
           <t>Health facility vehicle</t>
         </is>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Gari ya kituo cha afya</t>
+        </is>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="14.25">
       <c r="A15" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -2508,7 +2836,11 @@
           <t>Other</t>
         </is>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Nyenginezo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" selectLockedCells="1" sort="0" autoFilter="0" pivotTables="0" selectUnlockedCells="1"/>
@@ -2584,7 +2916,7 @@
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-11 17-29</v>
+        <v>2019-04-12 11-02</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fixing bugs found during internal testing of clinic-person-create form
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="60" count="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="64" count="64">
   <si>
     <t>type</t>
   </si>
@@ -114,6 +114,9 @@
     <t>Kitongoji:</t>
   </si>
   <si>
+    <t>string-length(translate(.," ","")) &gt;= 3</t>
+  </si>
+  <si>
     <t>house_number</t>
   </si>
   <si>
@@ -153,7 +156,16 @@
     <t>init</t>
   </si>
   <si>
+    <t>string-length(translate(.," ","")) &gt;= 2</t>
+  </si>
+  <si>
+    <t>Enter a first name</t>
+  </si>
+  <si>
     <t>ASK: What is their family name?</t>
+  </si>
+  <si>
+    <t>Enter a family name</t>
   </si>
   <si>
     <t>select_one sex</t>
@@ -813,13 +825,21 @@
       <c r="E29" t="s">
         <v>19</v>
       </c>
+      <c r="I29" t="s">
+        <v>29</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Enter a Kitongoji</t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:17" customHeight="1" ht="13.5">
       <c r="A30" t="s">
         <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -834,6 +854,16 @@
       <c r="E30" t="s">
         <v>19</v>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>string-length(translate(.," ","")) &gt;= 1</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Enter a house number</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>Enter the entire house number separated by slashes</t>
@@ -847,10 +877,10 @@
     </row>
     <row r="31" spans="1:17" customHeight="1" ht="13.5">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -864,6 +894,16 @@
       </c>
       <c r="E31" t="s">
         <v>19</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt;= 120</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Enter a number between 1 and 120.  Please discuss with your supervisor if it is taking you more than two hours to reach a client's house.</t>
+        </is>
       </c>
     </row>
     <row r="32" spans="1:17" customHeight="1" ht="13.5">
@@ -896,7 +936,7 @@
         <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -914,6 +954,14 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>selected(${means_of_travel_house},"other")</t>
+        </is>
+      </c>
+      <c r="I33" t="s">
+        <v>29</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Enter a means of travel</t>
         </is>
       </c>
     </row>
@@ -952,12 +1000,12 @@
         <v>4</v>
       </c>
       <c r="B36" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:17" customHeight="1" ht="13.5">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1000,7 +1048,7 @@
         </is>
       </c>
       <c r="F38" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -1023,7 +1071,7 @@
         </is>
       </c>
       <c r="F39" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -1036,7 +1084,7 @@
         <v>10</v>
       </c>
       <c r="B40" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:17" customHeight="1" ht="13.5">
@@ -1044,7 +1092,7 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1085,7 +1133,7 @@
     </row>
     <row r="43" spans="1:17" customHeight="1" ht="13.5">
       <c r="A43" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1128,7 +1176,7 @@
         </is>
       </c>
       <c r="F44" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:17" customHeight="1" ht="13.5">
@@ -1186,7 +1234,7 @@
         <v>4</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1196,7 +1244,7 @@
     </row>
     <row r="48" spans="1:17" customHeight="1" ht="13.5">
       <c r="A48" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -1307,7 +1355,7 @@
         </is>
       </c>
       <c r="F51" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="52" spans="1:17" customHeight="1" ht="13.5">
@@ -1315,7 +1363,7 @@
         <v>10</v>
       </c>
       <c r="B52" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="53" spans="1:17" customHeight="1" ht="13.5">
@@ -1323,7 +1371,7 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="54" spans="1:17" customHeight="1" ht="13.5">
@@ -1331,15 +1379,15 @@
         <v>4</v>
       </c>
       <c r="B54" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F54" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="55" spans="1:17" customHeight="1" ht="13.5">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1359,9 +1407,19 @@
       <c r="E55" t="s">
         <v>19</v>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt;= 30</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Kayas can have between 1 and 30 members</t>
+        </is>
+      </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>Ask the person to list the names of all people who live in the house, and count to ensure that the number they provided is correct. Long term visitors to the house, such as a woman returning home for delivery, should not be counted â only people who are permanent residents of the house.</t>
+          <t>Ask the person to list the names of all people who live in the house, and count to ensure that the number they provided is correct. Long term visitors to the house, such as a woman returning home for delivery, should not be counted - only people who are permanent residents of the house.</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -1395,7 +1453,7 @@
         <v>10</v>
       </c>
       <c r="B57" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58" spans="1:17" customHeight="1" ht="13.5">
@@ -1403,20 +1461,20 @@
         <v>4</v>
       </c>
       <c r="B58" t="s">
+        <v>42</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Household Contact Information</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tarifa za mawasiliano za kaya</t>
+        </is>
+      </c>
+      <c r="F58" t="s">
         <v>41</v>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Household Contact Information</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Tarifa za mawasiliano za kaya</t>
-        </is>
-      </c>
-      <c r="F58" t="s">
-        <v>40</v>
       </c>
       <c r="G58" t="s">
         <v>14</v>
@@ -1444,6 +1502,12 @@
       <c r="E59" t="s">
         <v>19</v>
       </c>
+      <c r="I59" t="s">
+        <v>43</v>
+      </c>
+      <c r="J59" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="60" spans="1:17" customHeight="1" ht="13.5">
       <c r="A60" t="s">
@@ -1455,7 +1519,7 @@
         </is>
       </c>
       <c r="C60" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1465,6 +1529,12 @@
       <c r="E60" t="s">
         <v>19</v>
       </c>
+      <c r="I60" t="s">
+        <v>43</v>
+      </c>
+      <c r="J60" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="61" spans="1:17" customHeight="1" ht="13.5">
       <c r="A61" t="s">
@@ -1483,7 +1553,7 @@
     </row>
     <row r="62" spans="1:17" customHeight="1" ht="13.5">
       <c r="A62" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1506,7 +1576,7 @@
     </row>
     <row r="63" spans="1:17" customHeight="1" ht="13.5">
       <c r="A63" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1529,7 +1599,7 @@
     </row>
     <row r="64" spans="1:17" customHeight="1" ht="13.5">
       <c r="A64" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
@@ -1572,7 +1642,7 @@
     </row>
     <row r="65" spans="1:17" customHeight="1" ht="13.5">
       <c r="A65" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1599,7 +1669,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>. &lt;= date-time(decimal-date-time(today() - (12 * 365))) and . &gt;= date-time(decimal-date-time(today() - (100 * 365)))</t>
+          <t>. &lt;= date-time(decimal-date-time(today() - (12 * 365.25))) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25)))</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -1636,13 +1706,13 @@
         <v>19</v>
       </c>
       <c r="I66" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J66" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K66" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="67" spans="1:17" customHeight="1" ht="13.5">
@@ -1665,13 +1735,13 @@
         </is>
       </c>
       <c r="I67" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J67" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K67" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -1734,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="B71" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" spans="1:17" customHeight="1" ht="13.5">
@@ -1742,7 +1812,7 @@
         <v>4</v>
       </c>
       <c r="B72" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -1757,7 +1827,7 @@
         </is>
       </c>
       <c r="B73" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -1770,7 +1840,7 @@
         </is>
       </c>
       <c r="F73" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G73" t="s">
         <v>14</v>
@@ -1854,6 +1924,12 @@
       <c r="E77" t="s">
         <v>19</v>
       </c>
+      <c r="I77" t="s">
+        <v>43</v>
+      </c>
+      <c r="J77" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="78" spans="1:17" customHeight="1" ht="13.5">
       <c r="A78" t="s">
@@ -1863,7 +1939,7 @@
         <v>20</v>
       </c>
       <c r="C78" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -1873,6 +1949,12 @@
       <c r="E78" t="s">
         <v>19</v>
       </c>
+      <c r="I78" t="s">
+        <v>43</v>
+      </c>
+      <c r="J78" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="79" spans="1:17" customHeight="1" ht="13.5">
       <c r="A79" t="s">
@@ -1919,7 +2001,7 @@
     </row>
     <row r="82" spans="1:17" customHeight="1" ht="13.5">
       <c r="A82" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B82" t="s">
         <v>21</v>
@@ -1955,7 +2037,7 @@
     </row>
     <row r="84" spans="1:17" customHeight="1" ht="13.5">
       <c r="A84" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B84" t="s">
         <v>22</v>
@@ -1991,7 +2073,7 @@
     </row>
     <row r="86" spans="1:17" customHeight="1" ht="13.5">
       <c r="A86" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
@@ -2054,7 +2136,7 @@
     </row>
     <row r="88" spans="1:17" customHeight="1" ht="13.5">
       <c r="A88" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2097,7 +2179,7 @@
     </row>
     <row r="89" spans="1:17" customHeight="1" ht="13.5">
       <c r="A89" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2124,7 +2206,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>(selected(${is_under_5},"yes") and . &lt;= date-time(decimal-date-time(today())) and . &gt; date-time(decimal-date-time(today() - (5 * 365)))) or (${exact_dob_known_c}="yes" and . &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365))))</t>
+          <t>(selected(${is_under_5},"yes") and . &lt;= date-time(decimal-date-time(today())) and . &gt; date-time(decimal-date-time(today() - (5 * 365.25)))) or (${exact_dob_known_c}="yes" and . &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25))))</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -2192,7 +2274,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>if(selected(${exact_dob_known_c},"yes"),if(((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &lt; 5,1,0),if(selected(${is_under_5},"yes"),int(1),int(0)))</t>
+          <t>if(selected(${exact_dob_known_c},"yes"),if(((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365.25) &lt; 5,1,0),if(selected(${is_under_5},"yes"),int(1),int(0)))</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2356,7 @@
         </is>
       </c>
       <c r="B97" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="98" spans="1:17" customHeight="1" ht="13.5">
@@ -2282,7 +2364,7 @@
         <v>10</v>
       </c>
       <c r="B98" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="99" spans="1:17" customHeight="1" ht="13.5">
@@ -2310,10 +2392,10 @@
         <v>4</v>
       </c>
       <c r="B100" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F100" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="101" spans="1:17" customHeight="1" ht="13.5">
@@ -2324,7 +2406,7 @@
         <v>15</v>
       </c>
       <c r="C101" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="L101" t="s">
         <v>16</v>
@@ -2341,7 +2423,7 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="L102" t="inlineStr">
         <is>
@@ -2377,7 +2459,7 @@
         <v>13</v>
       </c>
       <c r="C104" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="L104" t="inlineStr">
         <is>
@@ -2448,7 +2530,7 @@
         <v>11</v>
       </c>
       <c r="B108" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -2466,7 +2548,7 @@
         <v>11</v>
       </c>
       <c r="B109" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -2484,7 +2566,7 @@
         <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -2502,7 +2584,7 @@
         <v>11</v>
       </c>
       <c r="B111" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -2540,7 +2622,7 @@
         <v>10</v>
       </c>
       <c r="B113" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -2588,63 +2670,63 @@
     </row>
     <row r="2" spans="1:4" ht="14.25">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.25">
       <c r="A3" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.25">
       <c r="A4" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.25">
       <c r="A5" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.25">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -2704,7 +2786,7 @@
     </row>
     <row r="9" spans="1:4" ht="14.25">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -2724,7 +2806,7 @@
     </row>
     <row r="10" spans="1:4" ht="14.25">
       <c r="A10" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -2744,7 +2826,7 @@
     </row>
     <row r="11" spans="1:4" ht="14.25">
       <c r="A11" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2846,7 @@
     </row>
     <row r="12" spans="1:4" ht="14.25">
       <c r="A12" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -2784,7 +2866,7 @@
     </row>
     <row r="13" spans="1:4" ht="14.25">
       <c r="A13" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -2804,7 +2886,7 @@
     </row>
     <row r="14" spans="1:4" ht="14.25">
       <c r="A14" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -2824,7 +2906,7 @@
     </row>
     <row r="15" spans="1:4" ht="14.25">
       <c r="A15" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -2916,7 +2998,7 @@
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-12 11-02</v>
+        <v>2019-04-15 15-43</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Added constraint message for time.
Added constraint message in Swahili for time in the correct column.
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -1529,8 +1529,8 @@
     <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.86328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="28.54296875" customWidth="1"/>
-    <col min="10" max="10" width="37.81640625" customWidth="1"/>
-    <col min="11" max="11" width="26.76953125" customWidth="1"/>
+    <col min="10" max="10" width="114.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="122.04296875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="56.26953125" customWidth="1"/>
     <col min="13" max="13" width="31.40625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="28.54296875" customWidth="1"/>
@@ -2019,7 +2019,7 @@
       <c r="J31" t="s">
         <v>120</v>
       </c>
-      <c r="M31" t="s">
+      <c r="K31" t="s">
         <v>369</v>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="C2" s="3" t="str">
         <f ca="1">TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-16 9-07</v>
+        <v>2019-04-16 9-26</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>347</v>

</xml_diff>

<commit_message>
Adjusting data validation for kitongoji and adding swahili constraint messages
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="65" count="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="66" count="66">
   <si>
     <t>type</t>
   </si>
@@ -180,16 +180,19 @@
     <t>Kitongoji:</t>
   </si>
   <si>
+    <t>string-length(translate(.," ","")) &gt;= 1</t>
+  </si>
+  <si>
+    <t>house_number</t>
+  </si>
+  <si>
+    <t>travel_time</t>
+  </si>
+  <si>
+    <t>means_of_travel_other</t>
+  </si>
+  <si>
     <t>string-length(translate(.," ","")) &gt;= 3</t>
-  </si>
-  <si>
-    <t>house_number</t>
-  </si>
-  <si>
-    <t>travel_time</t>
-  </si>
-  <si>
-    <t>means_of_travel_other</t>
   </si>
   <si>
     <t>clinic</t>
@@ -1962,7 +1965,12 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Enter a Kitongoji</t>
+          <t>Enter a kitongoji</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Jaza kitongoji</t>
         </is>
       </c>
     </row>
@@ -1986,14 +1994,17 @@
       <c r="E85" t="s">
         <v>19</v>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>string-length(translate(.," ","")) &gt;= 1</t>
-        </is>
+      <c r="I85" t="s">
+        <v>51</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
           <t>Enter a house number</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Jaza nambari ya nyumba</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -2094,7 +2105,7 @@
         </is>
       </c>
       <c r="I88" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -2162,7 +2173,7 @@
         <v>4</v>
       </c>
       <c r="B92" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="93" spans="1:17" customHeight="1" ht="13.5">
@@ -2173,7 +2184,7 @@
         <v>15</v>
       </c>
       <c r="C93" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L93" t="s">
         <v>16</v>
@@ -2190,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="C94" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L94" t="inlineStr">
         <is>
@@ -2226,7 +2237,7 @@
         <v>13</v>
       </c>
       <c r="C96" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="L96" t="inlineStr">
         <is>
@@ -2333,7 +2344,7 @@
         <v>11</v>
       </c>
       <c r="B102" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -2438,7 +2449,7 @@
         <v>10</v>
       </c>
       <c r="B110" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2486,63 +2497,63 @@
     </row>
     <row r="2" spans="1:4" ht="14.75">
       <c r="A2" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.75">
       <c r="A3" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.75">
       <c r="A4" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.75">
       <c r="A5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" t="s">
         <v>64</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.75">
       <c r="A6" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -2602,7 +2613,7 @@
     </row>
     <row r="9" spans="1:4" ht="14.75">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2633,7 @@
     </row>
     <row r="10" spans="1:4" ht="14.75">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -2642,7 +2653,7 @@
     </row>
     <row r="11" spans="1:4" ht="14.75">
       <c r="A11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -2662,7 +2673,7 @@
     </row>
     <row r="12" spans="1:4" ht="14.75">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -2682,7 +2693,7 @@
     </row>
     <row r="13" spans="1:4" ht="14.75">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -2702,7 +2713,7 @@
     </row>
     <row r="14" spans="1:4" ht="14.75">
       <c r="A14" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -2722,7 +2733,7 @@
     </row>
     <row r="15" spans="1:4" ht="14.75">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -2814,7 +2825,7 @@
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-16 15-15</v>
+        <v>2019-04-17 11-30</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Adding start and end timestamps to all docs from clinic-create
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="66" count="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="68" count="68">
   <si>
     <t>type</t>
   </si>
@@ -102,6 +102,12 @@
     <t>meta</t>
   </si>
   <si>
+    <t>start</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
     <t>created_by</t>
   </si>
   <si>
@@ -192,13 +198,13 @@
     <t>means_of_travel_other</t>
   </si>
   <si>
+    <t>end_registration_note</t>
+  </si>
+  <si>
     <t>clinic</t>
   </si>
   <si>
     <t>NO_LABEL</t>
-  </si>
-  <si>
-    <t>geolocation</t>
   </si>
   <si>
     <t>means_of_travel</t>
@@ -312,7 +318,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q109"/>
+  <dimension ref="A1:Q115"/>
   <sheetFormatPr defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" style="0" width="26.863281249999996" bestFit="1" customWidth="1"/>
@@ -809,24 +815,18 @@
     </row>
     <row r="27" spans="1:17" ht="13.5">
       <c r="A27" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>25</v>
       </c>
-      <c r="L27" t="s">
-        <v>26</v>
-      </c>
     </row>
     <row r="28" spans="1:17" ht="13.5">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>27</v>
-      </c>
-      <c r="L28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="13.5">
@@ -834,434 +834,426 @@
         <v>11</v>
       </c>
       <c r="B29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L29" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="13.5">
       <c r="A30" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" t="s">
+        <v>29</v>
+      </c>
+      <c r="L30" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="13.5">
+      <c r="A31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" t="s">
+        <v>31</v>
+      </c>
+      <c r="L31" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="13.5">
+      <c r="A32" t="s">
         <v>10</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B32" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A31" t="s">
-        <v>10</v>
-      </c>
-      <c r="B31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A32" t="s">
-        <v>4</v>
-      </c>
-      <c r="B32" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:17" customHeight="1" ht="13.5">
       <c r="A33" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>num_hh_members</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>ASK: How many people live in your Kaya?</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>ULIZA: Ni watu wangapi wanaishi kwenye kaya yako?</t>
-        </is>
-      </c>
-      <c r="E33" t="s">
-        <v>19</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>. &gt; 0 and . &lt;= 30</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Kayas can have between 1 and 30 members</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Kaya iwe kati ya mtu 1 hadi watu 30.</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Ask the person to list the names of all people who live in the house, and count to ensure that the number they provided is correct. Long term visitors to the house, such as a woman returning home for delivery, should not be counted - only people who are permanent residents of the house.</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>Muombe mwenyeji wako aorodheshe majina ya watu wanaoishi kwenye kaya, na hesabu ili kuhakikisha idadi ni sawa. Usiwahesabu wageni walikokuja kutembea kwa muda mrefu, mfano wanawake walikuja nyumbani ili kujifungua, hesabu wakaazi wakudumu peke yao.</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:17" customHeight="1" ht="13.5">
       <c r="A34" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" t="s">
         <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>hh_repeat_note</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>SAY: For each person, I will ask some basic details about who they are, starting with the primary contact person for this household. Who should I list as the primary contact for this household, who will be the person I reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mtu ambaye naweza kuwasiliana naye kwenye nyumba hii. Je ni nani nimuorodheshe kama mtu wa kuwasiliana naye kwenye kaya hii ? Je, ni nani atakayekuwa mtu ninayeweza kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia? Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
-        </is>
       </c>
     </row>
     <row r="35" spans="1:17" customHeight="1" ht="13.5">
       <c r="A35" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>num_hh_members</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ASK: How many people live in your Kaya?</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni watu wangapi wanaishi kwenye kaya yako?</t>
+        </is>
+      </c>
+      <c r="E35" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt;= 30</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Kayas can have between 1 and 30 members</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Kaya iwe kati ya mtu 1 hadi watu 30.</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Ask the person to list the names of all people who live in the house, and count to ensure that the number they provided is correct. Long term visitors to the house, such as a woman returning home for delivery, should not be counted - only people who are permanent residents of the house.</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Muombe mwenyeji wako aorodheshe majina ya watu wanaoishi kwenye kaya, na hesabu ili kuhakikisha idadi ni sawa. Usiwahesabu wageni walikokuja kutembea kwa muda mrefu, mfano wanawake walikuja nyumbani ili kujifungua, hesabu wakaazi wakudumu peke yao.</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:17" customHeight="1" ht="13.5">
       <c r="A36" t="s">
-        <v>4</v>
-      </c>
-      <c r="B36" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>hh_repeat_note</t>
+        </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Household Contact Information</t>
+          <t>SAY: For each person, I will ask some basic details about who they are, starting with the primary contact person for this household. Who should I list as the primary contact for this household, who will be the person I reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Tarifa za mawasiliano za kaya</t>
-        </is>
-      </c>
-      <c r="G36" t="s">
-        <v>14</v>
+          <t>SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mtu ambaye naweza kuwasiliana naye kwenye nyumba hii. Je ni nani nimuorodheshe kama mtu wa kuwasiliana naye kwenye kaya hii ? Je, ni nani atakayekuwa mtu ninayeweza kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia? Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
+        </is>
       </c>
     </row>
     <row r="37" spans="1:17" customHeight="1" ht="13.5">
       <c r="A37" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>first_name_contact</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>ASK: What is the first name of the best contact person for your household?</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>ULIZA: ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
-        </is>
-      </c>
-      <c r="E37" t="s">
-        <v>19</v>
-      </c>
-      <c r="I37" t="s">
-        <v>36</v>
-      </c>
-      <c r="J37" t="s">
-        <v>37</v>
+        <v>10</v>
+      </c>
+      <c r="B37" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:17" customHeight="1" ht="13.5">
       <c r="A38" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>family_name_contact</t>
-        </is>
-      </c>
-      <c r="C38" t="s">
-        <v>38</v>
+        <v>4</v>
+      </c>
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Household Contact Information</t>
+        </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ULIZA: Ni lipi jina la babu yake?</t>
-        </is>
-      </c>
-      <c r="E38" t="s">
-        <v>19</v>
-      </c>
-      <c r="I38" t="s">
-        <v>36</v>
-      </c>
-      <c r="J38" t="s">
-        <v>39</v>
+          <t>Tarifa za mawasiliano za kaya</t>
+        </is>
+      </c>
+      <c r="G38" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:17" customHeight="1" ht="13.5">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>name_contact</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>concat(${first_name_contact}," ",${family_name_contact})</t>
-        </is>
+          <t>first_name_contact</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ASK: What is the first name of the best contact person for your household?</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ULIZA: ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
+        </is>
+      </c>
+      <c r="E39" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" t="s">
+        <v>38</v>
+      </c>
+      <c r="J39" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="40" spans="1:17" customHeight="1" ht="13.5">
       <c r="A40" t="s">
+        <v>37</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>family_name_contact</t>
+        </is>
+      </c>
+      <c r="C40" t="s">
         <v>40</v>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>sex_contact</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Enter ${first_name_contact}'s sex:</t>
-        </is>
-      </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Ingiza jinsia yake: </t>
+          <t>ULIZA: Ni lipi jina la babu yake?</t>
         </is>
       </c>
       <c r="E40" t="s">
         <v>19</v>
       </c>
+      <c r="I40" t="s">
+        <v>38</v>
+      </c>
+      <c r="J40" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="41" spans="1:17" customHeight="1" ht="13.5">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>11</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>exact_dob_known_contact</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>ASK: Do you know ${first_name_contact}'s exact date of birth?</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>ULIZA: Je unaijua tarehe sahihi yake ya  kuzaliwa? </t>
-        </is>
-      </c>
-      <c r="E41" t="s">
-        <v>19</v>
+          <t>name_contact</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>concat(${first_name_contact}," ",${family_name_contact})</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:17" customHeight="1" ht="13.5">
       <c r="A42" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>yob_contact</t>
+          <t>sex_contact</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ASK: In what year was ${first_name_contact} born?</t>
+          <t>Enter ${first_name_contact}'s sex:</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ULIZA Ni mwaka gani alizaliwa?</t>
+          <t>Ingiza jinsia yake: </t>
         </is>
       </c>
       <c r="E42" t="s">
         <v>19</v>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_contact},"no")</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>. &lt;= (format-date-time(today(),"%Y") - 12) and . &gt;= (format-date-time(today(),"%Y") - 100)</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Age must be between 12 and 100!</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Umri uwe ni kati ya 12 na 100!</t>
-        </is>
-      </c>
     </row>
     <row r="43" spans="1:17" customHeight="1" ht="13.5">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>dob_contact</t>
+          <t>exact_dob_known_contact</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ASK: What is ${first_name_contact}'s date of birth?</t>
+          <t>ASK: Do you know ${first_name_contact}'s exact date of birth?</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ULIZA: Je ni ipi tarehe yake kuzaliwa?</t>
+          <t>ULIZA: Je unaijua tarehe sahihi yake ya  kuzaliwa? </t>
         </is>
       </c>
       <c r="E43" t="s">
         <v>19</v>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_contact},"yes")</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>. &lt;= date-time(decimal-date-time(today() - (12 * 365.25))) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25)))</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Calculated age must be between 12 and 100!</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Umri uliohesabiwa ni lazima uwe kati ya miaka 12 na 100</t>
-        </is>
-      </c>
     </row>
     <row r="44" spans="1:17" customHeight="1" ht="13.5">
       <c r="A44" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>primary_phone_contact</t>
+          <t>yob_contact</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ASK: What is the best contact phone number for ${first_name_contact}?</t>
+          <t>ASK: In what year was ${first_name_contact} born?</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ULIZA: Je ni ipi nambari yake nzuri ya mawasilaano?</t>
+          <t>ULIZA Ni mwaka gani alizaliwa?</t>
         </is>
       </c>
       <c r="E44" t="s">
         <v>19</v>
       </c>
-      <c r="I44" t="s">
-        <v>43</v>
-      </c>
-      <c r="J44" t="s">
-        <v>44</v>
-      </c>
-      <c r="K44" t="s">
-        <v>45</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>selected(${exact_dob_known_contact},"no")</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>. &lt;= (format-date-time(today(),"%Y") - 12) and . &gt;= (format-date-time(today(),"%Y") - 100)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Age must be between 12 and 100!</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Umri uwe ni kati ya 12 na 100!</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:17" customHeight="1" ht="13.5">
       <c r="A45" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>secondary_phone_contact</t>
+          <t>dob_contact</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ASK: Is there another phone number used by ${first_name_contact} or another member of the household?</t>
+          <t>ASK: What is ${first_name_contact}'s date of birth?</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ULIZA: Je kuna nambari ya ziada anayotumia kuwasilaina?</t>
-        </is>
-      </c>
-      <c r="I45" t="s">
-        <v>43</v>
-      </c>
-      <c r="J45" t="s">
-        <v>44</v>
-      </c>
-      <c r="K45" t="s">
-        <v>45</v>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>You can leave this blank if there is only one good contact number for this household</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Unaweza acha pengo usijijaze chochote kama kuna nambari moja tu ya mawasiliano kwenye kaya hii</t>
+          <t>ULIZA: Je ni ipi tarehe yake kuzaliwa?</t>
+        </is>
+      </c>
+      <c r="E45" t="s">
+        <v>19</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>selected(${exact_dob_known_contact},"yes")</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>. &lt;= date-time(decimal-date-time(today() - (12 * 365.25))) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25)))</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Calculated age must be between 12 and 100!</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Umri uliohesabiwa ni lazima uwe kati ya miaka 12 na 100</t>
         </is>
       </c>
     </row>
     <row r="46" spans="1:17" customHeight="1" ht="13.5">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>dob_contact_calc</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>format-date(if(../dob_contact != '', ../dob_contact,concat(../yob_contact, '-01-01')), '%Y-%m-%d')</t>
-        </is>
+          <t>primary_phone_contact</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ASK: What is the best contact phone number for ${first_name_contact}?</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ULIZA: Je ni ipi nambari yake nzuri ya mawasilaano?</t>
+        </is>
+      </c>
+      <c r="E46" t="s">
+        <v>19</v>
+      </c>
+      <c r="I46" t="s">
+        <v>45</v>
+      </c>
+      <c r="J46" t="s">
+        <v>46</v>
+      </c>
+      <c r="K46" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:17" customHeight="1" ht="13.5">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>age_contact_years</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>(decimal-date-time(today()) - decimal-date-time(${dob_contact_calc})) div 365</t>
+          <t>secondary_phone_contact</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>ASK: Is there another phone number used by ${first_name_contact} or another member of the household?</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ULIZA: Je kuna nambari ya ziada anayotumia kuwasilaina?</t>
+        </is>
+      </c>
+      <c r="I47" t="s">
+        <v>45</v>
+      </c>
+      <c r="J47" t="s">
+        <v>46</v>
+      </c>
+      <c r="K47" t="s">
+        <v>47</v>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>You can leave this blank if there is only one good contact number for this household</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Unaweza acha pengo usijijaze chochote kama kuna nambari moja tu ya mawasiliano kwenye kaya hii</t>
         </is>
       </c>
     </row>
@@ -1271,263 +1263,257 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>reproductive_age_c</t>
+          <t>dob_contact_calc</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>if(selected(${sex_contact},"female") and ${age_contact_years} &gt;= 15 and ${age_contact_years} &lt;= 49,1,0)</t>
+          <t>format-date(if(../dob_contact != '', ../dob_contact,concat(../yob_contact, '-01-01')), '%Y-%m-%d')</t>
         </is>
       </c>
     </row>
     <row r="49" spans="1:17" customHeight="1" ht="13.5">
       <c r="A49" t="s">
-        <v>10</v>
-      </c>
-      <c r="B49" t="s">
-        <v>34</v>
+        <v>11</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>age_contact_years</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>(decimal-date-time(today()) - decimal-date-time(${dob_contact_calc})) div 365</t>
+        </is>
       </c>
     </row>
     <row r="50" spans="1:17" customHeight="1" ht="13.5">
       <c r="A50" t="s">
-        <v>4</v>
-      </c>
-      <c r="B50" t="s">
-        <v>46</v>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>${num_hh_members}&gt;1</t>
+        <v>11</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>reproductive_age_c</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>if(selected(${sex_contact},"female") and ${age_contact_years} &gt;= 15 and ${age_contact_years} &lt;= 49,1,0)</t>
         </is>
       </c>
     </row>
     <row r="51" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>begin repeat</t>
-        </is>
+      <c r="A51" t="s">
+        <v>10</v>
       </c>
       <c r="B51" t="s">
-        <v>47</v>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Household Member Information</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Taarifa za wanakaya</t>
-        </is>
-      </c>
-      <c r="G51" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>${num_hh_members}-1</t>
-        </is>
+        <v>36</v>
       </c>
     </row>
     <row r="52" spans="1:17" customHeight="1" ht="13.5">
       <c r="A52" t="s">
-        <v>33</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>hh_member_note</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Now, please enter information for the other members of the kaya.</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Sasa, tafadhali ingiza taarifa za watu wengine wanaoishi kwenye kaya.</t>
+        <v>4</v>
+      </c>
+      <c r="B52" t="s">
+        <v>48</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>${num_hh_members}&gt;1</t>
         </is>
       </c>
     </row>
     <row r="53" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A53" t="s">
-        <v>7</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>begin repeat</t>
+        </is>
       </c>
       <c r="B53" t="s">
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Household Member Information</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Taarifa za wanakaya</t>
+        </is>
       </c>
       <c r="G53" t="s">
-        <v>12</v>
-      </c>
-      <c r="P53" t="inlineStr">
-        <is>
-          <t>person</t>
+        <v>14</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>${num_hh_members}-1</t>
         </is>
       </c>
     </row>
     <row r="54" spans="1:17" customHeight="1" ht="13.5">
       <c r="A54" t="s">
-        <v>7</v>
-      </c>
-      <c r="B54" t="s">
-        <v>15</v>
-      </c>
-      <c r="G54" t="s">
-        <v>12</v>
-      </c>
-      <c r="L54" t="s">
-        <v>16</v>
-      </c>
-      <c r="P54" t="s">
-        <v>17</v>
+        <v>35</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>hh_member_note</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Now, please enter information for the other members of the kaya.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Sasa, tafadhali ingiza taarifa za watu wengine wanaoishi kwenye kaya.</t>
+        </is>
       </c>
     </row>
     <row r="55" spans="1:17" customHeight="1" ht="13.5">
       <c r="A55" t="s">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="B55" t="s">
-        <v>18</v>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>ASK: What is their first name?</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>ULIZA: Ni lipi jina lake la kwanza? </t>
-        </is>
-      </c>
-      <c r="E55" t="s">
-        <v>19</v>
-      </c>
-      <c r="I55" t="s">
-        <v>36</v>
-      </c>
-      <c r="J55" t="s">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="G55" t="s">
+        <v>12</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
       </c>
     </row>
     <row r="56" spans="1:17" customHeight="1" ht="13.5">
       <c r="A56" t="s">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="B56" t="s">
-        <v>20</v>
-      </c>
-      <c r="C56" t="s">
-        <v>38</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>ULIZA: Ni lipi jina lake la babu? </t>
-        </is>
-      </c>
-      <c r="E56" t="s">
-        <v>19</v>
-      </c>
-      <c r="I56" t="s">
-        <v>36</v>
-      </c>
-      <c r="J56" t="s">
-        <v>39</v>
+        <v>15</v>
+      </c>
+      <c r="G56" t="s">
+        <v>12</v>
+      </c>
+      <c r="L56" t="s">
+        <v>16</v>
+      </c>
+      <c r="P56" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:17" customHeight="1" ht="13.5">
       <c r="A57" t="s">
-        <v>11</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>first_name_c</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>../first_name</t>
-        </is>
+        <v>37</v>
+      </c>
+      <c r="B57" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>ASK: What is their first name?</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni lipi jina lake la kwanza? </t>
+        </is>
+      </c>
+      <c r="E57" t="s">
+        <v>19</v>
+      </c>
+      <c r="I57" t="s">
+        <v>38</v>
+      </c>
+      <c r="J57" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="58" spans="1:17" customHeight="1" ht="13.5">
       <c r="A58" t="s">
-        <v>11</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>family_name_c</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>../family_name</t>
-        </is>
+        <v>37</v>
+      </c>
+      <c r="B58" t="s">
+        <v>20</v>
+      </c>
+      <c r="C58" t="s">
+        <v>40</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni lipi jina lake la babu? </t>
+        </is>
+      </c>
+      <c r="E58" t="s">
+        <v>19</v>
+      </c>
+      <c r="I58" t="s">
+        <v>38</v>
+      </c>
+      <c r="J58" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="59" spans="1:17" customHeight="1" ht="13.5">
       <c r="A59" t="s">
         <v>11</v>
       </c>
-      <c r="B59" t="s">
-        <v>1</v>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>first_name_c</t>
+        </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>concat(${first_name_c}," ",${family_name_c})</t>
+          <t>../first_name</t>
         </is>
       </c>
     </row>
     <row r="60" spans="1:17" customHeight="1" ht="13.5">
       <c r="A60" t="s">
-        <v>40</v>
-      </c>
-      <c r="B60" t="s">
-        <v>21</v>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Enter ${first_name_c}'s sex</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Ingiza jinsia yake</t>
-        </is>
-      </c>
-      <c r="E60" t="s">
-        <v>19</v>
+        <v>11</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>family_name_c</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>../family_name</t>
+        </is>
       </c>
     </row>
     <row r="61" spans="1:17" customHeight="1" ht="13.5">
       <c r="A61" t="s">
         <v>11</v>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>sex_c</t>
-        </is>
+      <c r="B61" t="s">
+        <v>1</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>../sex</t>
+          <t>concat(${first_name_c}," ",${family_name_c})</t>
         </is>
       </c>
     </row>
     <row r="62" spans="1:17" customHeight="1" ht="13.5">
       <c r="A62" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B62" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ASK: Do you know ${first_name_c}'s exact date of birth?</t>
+          <t>Enter ${first_name_c}'s sex</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>ULIZA: Je unaijua terehe yake ya kuzaliwa kwa usahihi?</t>
+          <t>Ingiza jinsia yake</t>
         </is>
       </c>
       <c r="E62" t="s">
@@ -1540,95 +1526,68 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>exact_dob_known_c</t>
+          <t>sex_c</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>../exact_dob_known</t>
+          <t>../sex</t>
         </is>
       </c>
     </row>
     <row r="64" spans="1:17" customHeight="1" ht="13.5">
       <c r="A64" t="s">
-        <v>41</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>is_under_5</t>
-        </is>
+        <v>43</v>
+      </c>
+      <c r="B64" t="s">
+        <v>22</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ASK: Is ${first_name_c} under 5 years old?</t>
+          <t>ASK: Do you know ${first_name_c}'s exact date of birth?</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>ULIZA: Je mtoto yupo chini ya umri wa miaka 5?</t>
+          <t>ULIZA: Je unaijua terehe yake ya kuzaliwa kwa usahihi?</t>
         </is>
       </c>
       <c r="E64" t="s">
         <v>19</v>
       </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_c},"no")</t>
-        </is>
-      </c>
     </row>
     <row r="65" spans="1:17" customHeight="1" ht="13.5">
       <c r="A65" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>under_5_dob_note</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>SAY: For children under 5, I'd like to try and get some more specific information about their age. Can you try and remember the year and month when ${first_name_c} was born?</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>SEMA: Kwa watoto walio chini ya miaka 5 ningependa kupata taarifa zaidi kuhusu umri wao. Je,, unaweza kukumbuka ni mwezi na mwaka gani mtoto huyu alizaliwa?</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes")</t>
-        </is>
-      </c>
-      <c r="N65" t="inlineStr">
-        <is>
-          <t>It's important to try and get more exact age information for children. You can enter the child's date of birth as the first of the month in which they were born.</t>
-        </is>
-      </c>
-      <c r="O65" t="inlineStr">
-        <is>
-          <t>Ni muhimu kupata taarifa za uhakika kuhuru umri wa watoto. Unaweza kuingiza tarehe ya mwezi wa mtoto aliozaliwa</t>
+          <t>exact_dob_known_c</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>../exact_dob_known</t>
         </is>
       </c>
     </row>
     <row r="66" spans="1:17" customHeight="1" ht="13.5">
       <c r="A66" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>yob</t>
+          <t>is_under_5</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ASK: In what year was ${first_name_c} born?</t>
+          <t>ASK: Is ${first_name_c} under 5 years old?</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ULIZA: Ni mwaka gani alizaliwa?</t>
+          <t>ULIZA: Je mtoto yupo chini ya umri wa miaka 5?</t>
         </is>
       </c>
       <c r="E66" t="s">
@@ -1636,93 +1595,128 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"no")</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>format-date-time(today(),"%Y") - . &gt; 5 and format-date-time(today(),"%Y") - . &lt;= 100</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
-        <is>
-          <t>For children under 5 years of age, a more exact birthdate must be captured.</t>
-        </is>
-      </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
+          <t>selected(${exact_dob_known_c},"no")</t>
         </is>
       </c>
     </row>
     <row r="67" spans="1:17" customHeight="1" ht="13.5">
       <c r="A67" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>dob</t>
+          <t>under_5_dob_note</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ASK: What is ${first_name_c}'s date of birth?</t>
+          <t>SAY: For children under 5, I'd like to try and get some more specific information about their age. Can you try and remember the year and month when ${first_name_c} was born?</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ULIZA: Ipi ni tarehe yake kuzaliwa</t>
-        </is>
-      </c>
-      <c r="E67" t="s">
-        <v>19</v>
+          <t>SEMA: Kwa watoto walio chini ya miaka 5 ningependa kupata taarifa zaidi kuhusu umri wao. Je,, unaweza kukumbuka ni mwezi na mwaka gani mtoto huyu alizaliwa?</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>selected(${exact_dob_known_c},"yes") or (selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes"))</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>(selected(${is_under_5},"yes") and . &lt;= date-time(decimal-date-time(today())) and . &gt; date-time(decimal-date-time(today() - (5 * 365.25)))) or (${exact_dob_known_c}="yes" and . &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25))))</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>You've entered an invalid age - confirm that you've entered it properly.  For children under 5, confirm that the date is not more than 5 years ago.</t>
-        </is>
-      </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
+          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes")</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>It's important to try and get more exact age information for children. You can enter the child's date of birth as the first of the month in which they were born.</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Ni muhimu kupata taarifa za uhakika kuhuru umri wa watoto. Unaweza kuingiza tarehe ya mwezi wa mtoto aliozaliwa</t>
         </is>
       </c>
     </row>
     <row r="68" spans="1:17" customHeight="1" ht="13.5">
       <c r="A68" t="s">
-        <v>11</v>
-      </c>
-      <c r="B68" t="s">
-        <v>23</v>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>format-date(if(../dob != '', ../dob,concat(../yob, '-01-01')), '%Y-%m-%d')</t>
+        <v>34</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>yob</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ASK: In what year was ${first_name_c} born?</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ULIZA: Ni mwaka gani alizaliwa?</t>
+        </is>
+      </c>
+      <c r="E68" t="s">
+        <v>19</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>selected(${exact_dob_known_c},"no") and selected(${is_under_5},"no")</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>format-date-time(today(),"%Y") - . &gt; 5 and format-date-time(today(),"%Y") - . &lt;= 100</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>For children under 5 years of age, a more exact birthdate must be captured.</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
         </is>
       </c>
     </row>
     <row r="69" spans="1:17" customHeight="1" ht="13.5">
       <c r="A69" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>date_of_birth_c</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>../date_of_birth</t>
+          <t>dob</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>ASK: What is ${first_name_c}'s date of birth?</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ULIZA: Ipi ni tarehe yake kuzaliwa</t>
+        </is>
+      </c>
+      <c r="E69" t="s">
+        <v>19</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>selected(${exact_dob_known_c},"yes") or (selected(${exact_dob_known_c},"no") and selected(${is_under_5},"yes"))</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>(selected(${is_under_5},"yes") and . &lt;= date-time(decimal-date-time(today())) and . &gt; date-time(decimal-date-time(today() - (5 * 365.25)))) or (${exact_dob_known_c}="yes" and . &lt;= date-time(decimal-date-time(today())) and . &gt;= date-time(decimal-date-time(today() - (100 * 365.25))))</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>You've entered an invalid age - confirm that you've entered it properly.  For children under 5, confirm that the date is not more than 5 years ago.</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
         </is>
       </c>
     </row>
@@ -1730,14 +1724,12 @@
       <c r="A70" t="s">
         <v>11</v>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>reproductive_age</t>
-        </is>
+      <c r="B70" t="s">
+        <v>23</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>if(${sex_c}="female" and ((((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &gt;= 15 and ((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &lt;= 49)),int(1),int(0))</t>
+          <t>format-date(if(../dob != '', ../dob,concat(../yob, '-01-01')), '%Y-%m-%d')</t>
         </is>
       </c>
     </row>
@@ -1747,519 +1739,489 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>date_of_birth_c</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>../date_of_birth</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A72" t="s">
+        <v>11</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>reproductive_age</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>if(${sex_c}="female" and ((((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &gt;= 15 and ((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365) &lt;= 49)),int(1),int(0))</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A73" t="s">
+        <v>11</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>is_under_5_binary</t>
         </is>
       </c>
-      <c r="L71" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>if(selected(${exact_dob_known_c},"yes"),if(((decimal-date-time(today()) - decimal-date-time(${date_of_birth_c})) div 365.25) &lt; 5,1,0),if(selected(${is_under_5},"yes"),int(1),int(0)))</t>
         </is>
       </c>
     </row>
-    <row r="72" spans="1:17">
-      <c r="A72" t="s">
-        <v>33</v>
-      </c>
-      <c r="B72" t="inlineStr">
+    <row r="74" spans="1:17">
+      <c r="A74" t="s">
+        <v>35</v>
+      </c>
+      <c r="B74" t="inlineStr">
         <is>
           <t>return_children_note</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>SAY: From this registration, I've seen that you have a child under 5 who can benefit from this national program. Therefore, I'm asking for your permission to come back and check up on all issues related to their health care, nutrition, and child development. I would be grateful for your permission.</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>SEMA kutokanana usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe, na maendeleo yao. Nitafurahi kama nitapata ridhaa yenu.</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>${is_under_5_binary}=1</t>
         </is>
       </c>
     </row>
-    <row r="73" spans="1:17">
-      <c r="A73" t="s">
-        <v>33</v>
-      </c>
-      <c r="B73" t="inlineStr">
+    <row r="75" spans="1:17">
+      <c r="A75" t="s">
+        <v>35</v>
+      </c>
+      <c r="B75" t="inlineStr">
         <is>
           <t>return_women_note</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>SAY: I see that there are some women of reproductive age in your family. I'd like to ask your permission to return later to speak with them personally about issues related to health during pregnancy and childbirth.</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>SEMA: Nimeona kuna baadhi ya wanawake walio katika umri wa uzazi katika kaya yako. Ningeomba ridhaa yako kurudia ili kuja kuzungumza nao mambo muhimu ya afya kipindi cha ujauzito na baada ya kujifungua.</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>${reproductive_age} = 1 or ${reproductive_age_c} = 1</t>
         </is>
       </c>
-      <c r="G73" t="s">
+      <c r="G75" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A74" t="s">
-        <v>33</v>
-      </c>
-      <c r="B74" t="inlineStr">
+    <row r="76" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A76" t="s">
+        <v>35</v>
+      </c>
+      <c r="B76" t="inlineStr">
         <is>
           <t>debug_note</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>date of birth: ${date_of_birth_c} under_5_flag: ${is_under_5_binary} is reproductive age: ${reproductive_age}</t>
         </is>
       </c>
-      <c r="G74" t="s">
+      <c r="G76" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="75" spans="1:17" ht="13.5">
-      <c r="A75" t="s">
-        <v>4</v>
-      </c>
-      <c r="B75" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="76" spans="1:17" ht="13.5">
-      <c r="A76" t="s">
-        <v>11</v>
-      </c>
-      <c r="B76" t="s">
-        <v>25</v>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>../../../../name</t>
-        </is>
       </c>
     </row>
     <row r="77" spans="1:17" ht="13.5">
       <c r="A77" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B77" t="s">
-        <v>27</v>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>../../../../contact_id</t>
-        </is>
+        <v>24</v>
       </c>
     </row>
     <row r="78" spans="1:17" ht="13.5">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B78" t="s">
-        <v>29</v>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>../../../../facility_id</t>
-        </is>
+        <v>25</v>
       </c>
     </row>
     <row r="79" spans="1:17" ht="13.5">
       <c r="A79" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="B79" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="80" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>end repeat</t>
-        </is>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" ht="13.5">
+      <c r="A80" t="s">
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="81" spans="1:17" customHeight="1" ht="13.5">
+        <v>27</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>../../../../name</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:17" ht="13.5">
       <c r="A81" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>46</v>
+        <v>29</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>../../../../contact_id</t>
+        </is>
       </c>
     </row>
     <row r="82" spans="1:17" ht="13.5">
       <c r="A82" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>48</v>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Household Location</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Eneo la kaya</t>
-        </is>
-      </c>
-      <c r="G82" t="s">
-        <v>14</v>
+        <v>31</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>../../../../facility_id</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:17" ht="13.5">
       <c r="A83" t="s">
-        <v>33</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>intro_note</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>_The purpose of the following questions regarding the household location is to help you locate this house again when it is time to return for another visit to the people who live here. Enter the information that you will need to help you easily find this house again when you need to before you approach the household. What is the address of this household?_</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kuirudia tena. Kabla ya kuifika kaya hii. Ni ipi anuani ya nyumba hii?</t>
-        </is>
-      </c>
-      <c r="G83" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="84" spans="1:17" ht="13.5">
-      <c r="A84" t="s">
-        <v>35</v>
+        <v>10</v>
+      </c>
+      <c r="B83" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="84" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>end repeat</t>
+        </is>
       </c>
       <c r="B84" t="s">
         <v>49</v>
       </c>
-      <c r="C84" t="s">
-        <v>50</v>
-      </c>
-      <c r="D84" t="s">
-        <v>50</v>
-      </c>
-      <c r="E84" t="s">
-        <v>19</v>
-      </c>
-      <c r="I84" t="s">
-        <v>51</v>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>Enter a kitongoji</t>
-        </is>
-      </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>Jaza kitongoji</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" spans="1:17" ht="13.5">
+    </row>
+    <row r="85" spans="1:17" customHeight="1" ht="13.5">
       <c r="A85" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>52</v>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>House number:</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Nambari ya nyumba: </t>
-        </is>
-      </c>
-      <c r="E85" t="s">
-        <v>19</v>
-      </c>
-      <c r="I85" t="s">
-        <v>51</v>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>Enter a house number</t>
-        </is>
-      </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>Jaza nambari ya nyumba</t>
-        </is>
-      </c>
-      <c r="N85" t="inlineStr">
-        <is>
-          <t>Enter the entire house number separated by slashes</t>
-        </is>
-      </c>
-      <c r="O85" t="inlineStr">
-        <is>
-          <t>Ingiza nambari ya nyumba yote na tenganisha kwa kutumia alama ya Mkwaju</t>
-        </is>
+        <v>48</v>
       </c>
     </row>
     <row r="86" spans="1:17" ht="13.5">
       <c r="A86" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="B86" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>How many minutes does it take you to travel between this home and your home?</t>
+          <t>Household Location</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Ni dakika ngapi unatumia kutoka nyumbani kwenu hadi kwenye nyumba hii?</t>
-        </is>
-      </c>
-      <c r="E86" t="s">
-        <v>19</v>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>. &gt; 0 and . &lt;= 120</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>Enter a number between 1 and 120.  Please discuss with your supervisor if it is taking you more than two hours to reach a client's house.</t>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>Jaza nambari kati ya 1 na 120. Tafadhali zungumza na msimamizi wako kama inakuchukua masaa mawili kufika katika nyumba ya mteja wako. </t>
-        </is>
+          <t>Eneo la kaya</t>
+        </is>
+      </c>
+      <c r="G86" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="87" spans="1:17" ht="13.5">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>select_one means_of_travel</t>
-        </is>
+      <c r="A87" t="s">
+        <v>35</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>means_of_travel_house</t>
+          <t>intro_note</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>How do you travel between your home and this home?</t>
+          <t>_The purpose of the following questions regarding the household location is to help you locate this house again when it is time to return for another visit to the people who live here. Enter the information that you will need to help you easily find this house again when you need to before you approach the household. What is the address of this household?_</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Unatumia usafiri gani?</t>
-        </is>
-      </c>
-      <c r="E87" t="s">
-        <v>19</v>
+          <t>Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kuirudia tena. Kabla ya kuifika kaya hii. Ni ipi anuani ya nyumba hii?</t>
+        </is>
+      </c>
+      <c r="G87" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="88" spans="1:17" ht="13.5">
       <c r="A88" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B88" t="s">
-        <v>54</v>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Specify other means of travel:</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Taja aina nyengine ya usafiri: </t>
-        </is>
+        <v>51</v>
+      </c>
+      <c r="C88" t="s">
+        <v>52</v>
+      </c>
+      <c r="D88" t="s">
+        <v>52</v>
       </c>
       <c r="E88" t="s">
         <v>19</v>
       </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>selected(${means_of_travel_house},"other")</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>string-length(translate(.," ","")) &gt;= 3</t>
-        </is>
+      <c r="I88" t="s">
+        <v>53</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Enter a means of travel</t>
+          <t>Enter a kitongoji</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Jaza njia ya usafiri</t>
+          <t>Jaza kitongoji</t>
         </is>
       </c>
     </row>
     <row r="89" spans="1:17" ht="13.5">
       <c r="A89" t="s">
+        <v>37</v>
+      </c>
+      <c r="B89" t="s">
+        <v>54</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>House number:</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Nambari ya nyumba: </t>
+        </is>
+      </c>
+      <c r="E89" t="s">
+        <v>19</v>
+      </c>
+      <c r="I89" t="s">
+        <v>53</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Enter a house number</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Jaza nambari ya nyumba</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Enter the entire house number separated by slashes</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Ingiza nambari ya nyumba yote na tenganisha kwa kutumia alama ya Mkwaju</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" spans="1:17" ht="13.5">
+      <c r="A90" t="s">
+        <v>34</v>
+      </c>
+      <c r="B90" t="s">
+        <v>55</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>How many minutes does it take you to travel between this home and your home?</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Ni dakika ngapi unatumia kutoka nyumbani kwenu hadi kwenye nyumba hii?</t>
+        </is>
+      </c>
+      <c r="E90" t="s">
+        <v>19</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>. &gt; 0 and . &lt;= 120</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Enter a number between 1 and 120.  Please discuss with your supervisor if it is taking you more than two hours to reach a client's house.</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Jaza nambari kati ya 1 na 120. Tafadhali zungumza na msimamizi wako kama inakuchukua masaa mawili kufika katika nyumba ya mteja wako. </t>
+        </is>
+      </c>
+    </row>
+    <row r="91" spans="1:17" ht="13.5">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>select_one means_of_travel</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>means_of_travel_house</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>How do you travel between your home and this home?</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Unatumia usafiri gani?</t>
+        </is>
+      </c>
+      <c r="E91" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="92" spans="1:17" ht="13.5">
+      <c r="A92" t="s">
+        <v>37</v>
+      </c>
+      <c r="B92" t="s">
+        <v>56</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Specify other means of travel:</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Taja aina nyengine ya usafiri: </t>
+        </is>
+      </c>
+      <c r="E92" t="s">
+        <v>19</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>selected(${means_of_travel_house},"other")</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>string-length(translate(.," ","")) &gt;= 3</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Enter a means of travel</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Jaza njia ya usafiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" spans="1:17" ht="13.5">
+      <c r="A93" t="s">
         <v>10</v>
       </c>
-      <c r="B89" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="90" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A90" t="s">
-        <v>33</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>end_registration_note</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>_The registration process for this kaya is now complete._</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>_Mchakato wa usajili katika kaya umekamilika_</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A91" t="s">
-        <v>4</v>
-      </c>
-      <c r="B91" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="92" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A92" t="s">
-        <v>11</v>
-      </c>
-      <c r="B92" t="s">
-        <v>15</v>
-      </c>
-      <c r="C92" t="s">
-        <v>56</v>
-      </c>
-      <c r="L92" t="s">
-        <v>16</v>
-      </c>
-      <c r="P92" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="93" spans="1:17" customHeight="1" ht="13.5">
-      <c r="A93" t="s">
-        <v>11</v>
-      </c>
       <c r="B93" t="s">
-        <v>1</v>
-      </c>
-      <c r="C93" t="s">
-        <v>56</v>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>concat(../../contact/first_name,../../contact/last_name, ' Household')</t>
-        </is>
+        <v>50</v>
       </c>
     </row>
     <row r="94" spans="1:17" customHeight="1" ht="13.5">
       <c r="A94" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="B94" t="s">
         <v>57</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>concat(../../inputs/meta/location/lat, concat(' ', ../../inputs/meta/location/long))</t>
+          <t>_The registration process for this kaya is now complete._</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>_Mchakato wa usajili katika kaya umekamilika_</t>
         </is>
       </c>
     </row>
     <row r="95" spans="1:17" customHeight="1" ht="13.5">
       <c r="A95" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B95" t="s">
-        <v>13</v>
-      </c>
-      <c r="C95" t="s">
-        <v>56</v>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>"NEW"</t>
-        </is>
+        <v>58</v>
       </c>
     </row>
     <row r="96" spans="1:17" customHeight="1" ht="13.5">
       <c r="A96" t="s">
         <v>11</v>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>household_district</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>District</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>${district_auto}</t>
-        </is>
+      <c r="B96" t="s">
+        <v>15</v>
+      </c>
+      <c r="C96" t="s">
+        <v>59</v>
+      </c>
+      <c r="L96" t="s">
+        <v>16</v>
+      </c>
+      <c r="P96" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="97" spans="1:17" customHeight="1" ht="13.5">
       <c r="A97" t="s">
         <v>11</v>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>household_shehia</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>Shehia</t>
-        </is>
+      <c r="B97" t="s">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>59</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>${shehia_auto}</t>
+          <t>concat(../../contact/first_name,../../contact/last_name, ' Household')</t>
         </is>
       </c>
     </row>
@@ -2267,17 +2229,19 @@
       <c r="A98" t="s">
         <v>11</v>
       </c>
-      <c r="B98" t="s">
-        <v>49</v>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>geolocation</t>
+        </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Kitongoji</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>../../household_location/kitongoji</t>
+          <t>concat(../../inputs/meta/location/lat, concat(' ', ../../inputs/meta/location/long))</t>
         </is>
       </c>
     </row>
@@ -2286,16 +2250,14 @@
         <v>11</v>
       </c>
       <c r="B99" t="s">
-        <v>52</v>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Household number</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="C99" t="s">
+        <v>59</v>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>../../household_location/house_number</t>
+          <t>"NEW"</t>
         </is>
       </c>
     </row>
@@ -2303,17 +2265,19 @@
       <c r="A100" t="s">
         <v>11</v>
       </c>
-      <c r="B100" t="s">
-        <v>53</v>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>household_district</t>
+        </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Time from home to household (minutes)</t>
+          <t>District</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>../../household_location/travel_time</t>
+          <t>${district_auto}</t>
         </is>
       </c>
     </row>
@@ -2321,17 +2285,19 @@
       <c r="A101" t="s">
         <v>11</v>
       </c>
-      <c r="B101" t="s">
-        <v>58</v>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>household_shehia</t>
+        </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Means of travel to household</t>
+          <t>Shehia</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>../../household_location/means_of_travel_house</t>
+          <t>${shehia_auto}</t>
         </is>
       </c>
     </row>
@@ -2340,16 +2306,16 @@
         <v>11</v>
       </c>
       <c r="B102" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Other means of travel to household</t>
+          <t>Kitongoji</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>../../household_location/means_of_travel_other</t>
+          <t>../../household_location/kitongoji</t>
         </is>
       </c>
     </row>
@@ -2357,77 +2323,165 @@
       <c r="A103" t="s">
         <v>11</v>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" t="s">
+        <v>54</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Household number</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>../../household_location/house_number</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A104" t="s">
+        <v>11</v>
+      </c>
+      <c r="B104" t="s">
+        <v>55</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Time from home to household (minutes)</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>../../household_location/travel_time</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A105" t="s">
+        <v>11</v>
+      </c>
+      <c r="B105" t="s">
+        <v>60</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Means of travel to household</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>../../household_location/means_of_travel_house</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A106" t="s">
+        <v>11</v>
+      </c>
+      <c r="B106" t="s">
+        <v>56</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Other means of travel to household</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>../../household_location/means_of_travel_other</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A107" t="s">
+        <v>11</v>
+      </c>
+      <c r="B107" t="inlineStr">
         <is>
           <t>number_hh_members</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Number of members of hosuehold</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr">
+      <c r="L107" t="inlineStr">
         <is>
           <t>../../household_member_count/num_household_members</t>
         </is>
-      </c>
-    </row>
-    <row r="104" spans="1:17" ht="13.5">
-      <c r="A104" t="s">
-        <v>4</v>
-      </c>
-      <c r="B104" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="105" spans="1:17" ht="13.5">
-      <c r="A105" t="s">
-        <v>11</v>
-      </c>
-      <c r="B105" t="s">
-        <v>25</v>
-      </c>
-      <c r="L105" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="106" spans="1:17" ht="13.5">
-      <c r="A106" t="s">
-        <v>11</v>
-      </c>
-      <c r="B106" t="s">
-        <v>27</v>
-      </c>
-      <c r="L106" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="107" spans="1:17" ht="13.5">
-      <c r="A107" t="s">
-        <v>11</v>
-      </c>
-      <c r="B107" t="s">
-        <v>29</v>
-      </c>
-      <c r="L107" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="108" spans="1:17" ht="13.5">
       <c r="A108" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B108" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="109" spans="1:17" customHeight="1" ht="13.5">
+    <row r="109" spans="1:17" ht="13.5">
       <c r="A109" t="s">
+        <v>25</v>
+      </c>
+      <c r="B109" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="110" spans="1:17" ht="13.5">
+      <c r="A110" t="s">
+        <v>26</v>
+      </c>
+      <c r="B110" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="111" spans="1:17" ht="13.5">
+      <c r="A111" t="s">
+        <v>11</v>
+      </c>
+      <c r="B111" t="s">
+        <v>27</v>
+      </c>
+      <c r="L111" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="112" spans="1:17" ht="13.5">
+      <c r="A112" t="s">
+        <v>11</v>
+      </c>
+      <c r="B112" t="s">
+        <v>29</v>
+      </c>
+      <c r="L112" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="113" spans="1:17" ht="13.5">
+      <c r="A113" t="s">
+        <v>11</v>
+      </c>
+      <c r="B113" t="s">
+        <v>31</v>
+      </c>
+      <c r="L113" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="114" spans="1:17" ht="13.5">
+      <c r="A114" t="s">
         <v>10</v>
       </c>
-      <c r="B109" t="s">
-        <v>55</v>
+      <c r="B114" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="115" spans="1:17" customHeight="1" ht="13.5">
+      <c r="A115" t="s">
+        <v>10</v>
+      </c>
+      <c r="B115" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2475,63 +2529,63 @@
     </row>
     <row r="2" spans="1:4" ht="14.75">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="14.75">
       <c r="A3" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="14.75">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="14.75">
       <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.75">
       <c r="A6" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -2591,7 +2645,7 @@
     </row>
     <row r="9" spans="1:4" ht="14.75">
       <c r="A9" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -2611,7 +2665,7 @@
     </row>
     <row r="10" spans="1:4" ht="14.75">
       <c r="A10" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -2631,7 +2685,7 @@
     </row>
     <row r="11" spans="1:4" ht="14.75">
       <c r="A11" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -2651,7 +2705,7 @@
     </row>
     <row r="12" spans="1:4" ht="14.75">
       <c r="A12" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -2671,7 +2725,7 @@
     </row>
     <row r="13" spans="1:4" ht="14.75">
       <c r="A13" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -2691,7 +2745,7 @@
     </row>
     <row r="14" spans="1:4" ht="14.75">
       <c r="A14" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2765,7 @@
     </row>
     <row r="15" spans="1:4" ht="14.75">
       <c r="A15" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -2803,7 +2857,7 @@
       </c>
       <c r="C2" s="3" t="str">
         <f>TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-04-23 10-49</v>
+        <v>2019-05-06 16-27</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Changed the introductory HH registration text and fixed lower case issue (#11)
* Changed the introductory HH registration text

* Made changes to the XML
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" state="visible" r:id="rId2"/>
@@ -314,10 +314,10 @@
     <t xml:space="preserve">hh_repeat_note</t>
   </si>
   <si>
-    <t xml:space="preserve">SAY: For each person, I will ask some basic details about who they are, starting with the primary contact person for this household. Who should I list as the primary contact for this household, who will be the person I reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mtu ambaye naweza kuwasiliana naye kwenye nyumba hii. Je ni nani nimuorodheshe kama mtu wa kuwasiliana naye kwenye kaya hii ? Je, ni nani atakayekuwa mtu ninayeweza kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia? Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
+    <t xml:space="preserve">SAY: For each person, I will ask some basic details about who they are, starting with either the head of household or best contact person for this household. Who should I list as the person I can reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mkuu wa kaya au mtu mzima yoyote ambaye naweza kuwasiliana naye kwenye nyumba hii. Je, ni nani atakayekuwa mtu ninayeweza  kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia?  Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
   </si>
   <si>
     <t xml:space="preserve">init</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">ASK: What is the first name of the best contact person for your household?</t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
+    <t xml:space="preserve">ULIZA: Ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
   </si>
   <si>
     <t xml:space="preserve">string-length(translate(.," ","")) &gt;= 2</t>
@@ -1020,6 +1020,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1145,9 +1146,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="32.62"/>
@@ -1156,7 +1157,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="64.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="35.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="32.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="9.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="26.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="18" style="1" width="10.45"/>
   </cols>
@@ -2804,7 +2805,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1.66666666666667" bottom="1.66666666666667" header="1" footer="1"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="atEnd" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Sans,Regular"&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Sans,Regular"Page &amp;P</oddFooter>
@@ -3040,7 +3041,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1.66666666666667" bottom="1.66666666666667" header="1" footer="1"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="atEnd" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Sans,Regular"&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Sans,Regular"Page &amp;P</oddFooter>
@@ -3060,7 +3061,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="7" style="1" width="10.45"/>
   </cols>
@@ -3094,7 +3095,7 @@
       </c>
       <c r="C2" s="4" t="str">
         <f aca="true">TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-05-16  10-10</v>
+        <v>2019-05-17  16-05</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>323</v>
@@ -3107,7 +3108,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1.66666666666667" bottom="1.66666666666667" header="1" footer="1"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="atEnd" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Sans,Regular"&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Sans,Regular"Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
Household title translation (#13)
* Added swahili translation for household title

* Resolved merge conflict
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -788,7 +788,7 @@
     <t xml:space="preserve">clinic</t>
   </si>
   <si>
-    <t xml:space="preserve">concat(../../contact/first_name,../../contact/last_name, ' Household')</t>
+    <t xml:space="preserve">concat('Nyumba ya ' , ../../contact/first_name,../../contact/last_name, '  - Nyumba no. ',../../household_location/house_number)</t>
   </si>
   <si>
     <t xml:space="preserve">geolocation</t>
@@ -1148,7 +1148,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="32.62"/>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="C2" s="4" t="str">
         <f aca="true">TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-05-17  16-05</v>
+        <v>2019-05-20  10-59</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>323</v>

</xml_diff>

<commit_message>
Household age bug (#15)
* Modified translations and fixed age related bug

* Compiled clinic create xml

* Changed age related error msg

* Changed the error msg related to age
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="330">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -389,25 +389,34 @@
     <t xml:space="preserve">ULIZA: Je unaijua tarehe sahihi yake ya  kuzaliwa? </t>
   </si>
   <si>
+    <t xml:space="preserve">age_estimate_contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASK: What is ${first_name_contact}'s estimated age in years? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULIZA: Je kwa makadirio ${first_name_contact} ana miaka mingapi? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${exact_dob_known_contact} = “no”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">. &gt;= 12 and . &lt;= 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age must be between 12 and 100!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umri uwe ni kati ya 12 na 100!</t>
+  </si>
+  <si>
     <t xml:space="preserve">yob_contact</t>
   </si>
   <si>
-    <t xml:space="preserve">ASK: In what year was ${first_name_contact} born?</t>
-  </si>
-  <si>
     <t xml:space="preserve">ULIZA Ni mwaka gani alizaliwa?</t>
   </si>
   <si>
-    <t xml:space="preserve">selected(${exact_dob_known_contact},"no")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">. &lt;= (format-date-time(today(),"%Y") - 12) and . &gt;= (format-date-time(today(),"%Y") - 100)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age must be between 12 and 100!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Umri uwe ni kati ya 12 na 100!</t>
+    <t xml:space="preserve">format-date-time(today(),"%Y")  - ../age_estimate_contact</t>
   </si>
   <si>
     <t xml:space="preserve">date</t>
@@ -509,10 +518,10 @@
     <t xml:space="preserve">hh_member_note</t>
   </si>
   <si>
-    <t xml:space="preserve">Now, please enter information for the other members of the kaya.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sasa, tafadhali ingiza taarifa za watu wengine wanaoishi kwenye kaya.</t>
+    <t xml:space="preserve">Now, please enter information for the next member of the kaya.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sasa, tafadhali ingiza taarifa za mtu anayefuata katika kaya yako.</t>
   </si>
   <si>
     <t xml:space="preserve">person</t>
@@ -566,25 +575,31 @@
     <t xml:space="preserve">../exact_dob_known</t>
   </si>
   <si>
+    <t xml:space="preserve">age_estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASK: Do you know ${first_name_c}'s estimated age in years? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULIZA: Je kwa makadirio ${first_name_c} ana miaka mingapi? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">${exact_dob_known_c}="no"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">. &gt; 5 and . &lt;= 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Age must be between 5 and 100. For children under 5 years of age, a more exact birthdate must be captured.  Please select "Yes" to the prior question and do your best to capture more exact birthdate information about the child.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umri lazime uwe kati ya miaka 5 hadi miaka 100. Kwa watoto walio chini ya umri wa miaka 5, tarehe yao ya kuzaliwa nilazima ichukuliwe.</t>
+  </si>
+  <si>
     <t xml:space="preserve">yob</t>
   </si>
   <si>
-    <t xml:space="preserve">ASK: In what year was ${first_name_c} born?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ULIZA: Ni mwaka gani alizaliwa?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${exact_dob_known_c}="no"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">format-date-time(today(),"%Y") - . &gt; 5 and format-date-time(today(),"%Y") - . &lt;= 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For children under 5 years of age, a more exact birthdate must be captured.  Please select "Yes" to the prior question and do your best to capture more exact birthdate information about the child.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kwa watoto walio chini ya umri wa miaka 5, tarehe yake yao ya kuzaliwa nilazima ichukuliwe.</t>
+    <t xml:space="preserve">format-date-time(today(),"%Y")  - ../age_estimate</t>
   </si>
   <si>
     <t xml:space="preserve">dob</t>
@@ -686,7 +701,7 @@
     <t xml:space="preserve">_The purpose of the following questions regarding the household location is to help you locate this house again when it is time to return for another visit to the people who live here. Enter the information that you will need to help you easily find this house again when you need to before you approach the household. What is the address of this household?_</t>
   </si>
   <si>
-    <t xml:space="preserve">Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kuirudia tena. Kabla ya kuifika kaya hii. Ni ipi anuani ya nyumba hii?</t>
+    <t xml:space="preserve">Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kuirudia tena. Ni ipi anuani ya nyumba hii?</t>
   </si>
   <si>
     <t xml:space="preserve">kitongoji</t>
@@ -1102,13 +1117,21 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1140,18 +1163,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:Q1048576"/>
   <sheetFormatPr defaultRowHeight="13" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="33.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="324.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="54.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="56.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="32.62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="133.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="131.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="139.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="64.31"/>
@@ -1783,7 +1806,7 @@
       <c r="A42" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="2" t="s">
         <v>119</v>
       </c>
       <c r="C42" s="1" t="s">
@@ -1810,57 +1833,47 @@
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="D43" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C43" s="1" t="s">
+      <c r="J43" s="0"/>
+      <c r="K43" s="0"/>
+      <c r="L43" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F43" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="I43" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="J43" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="F44" s="1" t="s">
+        <v>133</v>
+      </c>
       <c r="I44" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1868,39 +1881,54 @@
         <v>99</v>
       </c>
       <c r="B45" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="J45" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="K45" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="N45" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="O45" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="B46" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="L46" s="1" t="s">
+      <c r="I46" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="K46" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="N46" s="1" t="s">
         <v>146</v>
+      </c>
+      <c r="O46" s="1" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1908,10 +1936,10 @@
         <v>30</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1919,83 +1947,77 @@
         <v>30</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>96</v>
+        <v>152</v>
+      </c>
+      <c r="L49" s="1" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F50" s="1" t="s">
-        <v>152</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>153</v>
+        <v>17</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>154</v>
       </c>
       <c r="C51" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q51" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="D52" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D52" s="1" t="s">
+      <c r="G52" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q52" s="1" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P53" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2003,7 +2025,7 @@
         <v>21</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>19</v>
@@ -2011,34 +2033,28 @@
       <c r="G54" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L54" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="P54" s="1" t="s">
-        <v>43</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>104</v>
+        <v>19</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="P55" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2046,13 +2062,13 @@
         <v>99</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>106</v>
+        <v>165</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>47</v>
@@ -2061,18 +2077,30 @@
         <v>103</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="L57" s="1" t="s">
-        <v>166</v>
+        <v>49</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2080,10 +2108,10 @@
         <v>30</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2091,146 +2119,150 @@
         <v>30</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>1</v>
+        <v>170</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>30</v>
+        <v>111</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="L61" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C61" s="1" t="s">
         <v>173</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>115</v>
+        <v>30</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="D62" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="E62" s="1" t="s">
-        <v>47</v>
+      <c r="L62" s="1" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="L63" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C63" s="1" t="s">
         <v>177</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="C64" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="L64" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="E64" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="I64" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="K64" s="1" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>185</v>
+        <v>83</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>47</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="K65" s="1" t="s">
-        <v>191</v>
-      </c>
+        <v>187</v>
+      </c>
+      <c r="L65" s="0"/>
     </row>
     <row r="66" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="L66" s="1" t="s">
-        <v>192</v>
+      <c r="B66" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L66" s="3" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>30</v>
+        <v>129</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F67" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="L67" s="1" t="s">
+      <c r="I67" s="1" t="s">
         <v>194</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2238,10 +2270,10 @@
         <v>30</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>195</v>
+        <v>63</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2249,94 +2281,94 @@
         <v>30</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="C70" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="D70" s="1" t="s">
+      <c r="L70" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F70" s="1" t="s">
+    </row>
+    <row r="71" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="71" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B71" s="1" t="s">
+      <c r="L71" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C71" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="72" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F72" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="C72" s="1" t="s">
+    </row>
+    <row r="73" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B73" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="G72" s="1" t="s">
+      <c r="C73" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G73" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="L74" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L75" s="1" t="s">
-        <v>210</v>
+        <v>75</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2344,276 +2376,270 @@
         <v>30</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="L76" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>78</v>
+      </c>
+      <c r="L77" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>212</v>
+        <v>30</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>80</v>
+      </c>
+      <c r="L78" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>17</v>
+        <v>217</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="G80" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="G81" s="1" t="s">
-        <v>40</v>
+        <v>154</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>99</v>
+        <v>17</v>
       </c>
       <c r="B82" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>219</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>220</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="E82" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I82" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="J82" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>223</v>
+      <c r="G82" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="E83" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I83" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="J83" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="N83" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="O83" s="1" t="s">
-        <v>230</v>
+        <v>223</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>47</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>237</v>
+        <v>99</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="86" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I85" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="J85" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="N85" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="O85" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F86" s="1" t="s">
-        <v>244</v>
-      </c>
       <c r="I86" s="1" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="J88" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="K88" s="1" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B87" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="B89" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>19</v>
+        <v>218</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>41</v>
+        <v>253</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L90" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="P90" s="1" t="s">
-        <v>43</v>
+        <v>254</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>1</v>
+        <v>256</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="L91" s="1" t="s">
-        <v>252</v>
-      </c>
     </row>
     <row r="92" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>253</v>
+        <v>41</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>254</v>
+        <v>19</v>
       </c>
       <c r="L92" s="1" t="s">
-        <v>255</v>
+        <v>42</v>
+      </c>
+      <c r="P92" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,13 +2647,13 @@
         <v>30</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="C93" s="1" t="s">
         <v>19</v>
       </c>
       <c r="L93" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2635,13 +2661,13 @@
         <v>30</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L94" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2649,13 +2675,13 @@
         <v>30</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>260</v>
+        <v>39</v>
       </c>
       <c r="C95" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L95" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="L95" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2663,7 +2689,7 @@
         <v>30</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>219</v>
+        <v>262</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>263</v>
@@ -2677,13 +2703,13 @@
         <v>30</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>224</v>
+        <v>265</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2691,13 +2717,13 @@
         <v>30</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L98" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2705,7 +2731,7 @@
         <v>30</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>269</v>
+        <v>229</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>270</v>
@@ -2719,7 +2745,7 @@
         <v>30</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="C100" s="1" t="s">
         <v>272</v>
@@ -2742,37 +2768,43 @@
         <v>276</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>75</v>
+        <v>246</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+      <c r="L102" s="1" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>76</v>
+        <v>279</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>280</v>
       </c>
       <c r="L103" s="1" t="s">
-        <v>77</v>
+        <v>281</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L104" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2780,28 +2812,51 @@
         <v>30</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="L105" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L106" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="L107" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B106" s="1" t="s">
+      <c r="B108" s="1" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A107" s="1" t="s">
+    <row r="109" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B107" s="1" t="s">
-        <v>251</v>
-      </c>
-    </row>
+      <c r="B109" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1.66666666666667" bottom="1.66666666666667" header="1" footer="1"/>
@@ -2829,213 +2884,213 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B1" s="2" t="s">
+      <c r="A1" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>280</v>
+      <c r="C2" s="5" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="A3" s="5" t="s">
         <v>283</v>
       </c>
+      <c r="B3" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>279</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>282</v>
+      <c r="A5" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>287</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>286</v>
+      <c r="A6" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>291</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>289</v>
+      <c r="B7" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>294</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>292</v>
+      <c r="B8" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>297</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>294</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>295</v>
+      <c r="A9" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>298</v>
+      <c r="A10" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>303</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>301</v>
+      <c r="A11" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>306</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>304</v>
+      <c r="A12" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>309</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>307</v>
+      <c r="A13" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>312</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>310</v>
+      <c r="A14" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>315</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>313</v>
+      <c r="A15" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>317</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>318</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
   </sheetData>
@@ -3067,43 +3122,43 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>320</v>
       </c>
+      <c r="B1" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="C2" s="4" t="str">
+      <c r="A2" s="5" t="s">
+        <v>326</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="C2" s="6" t="str">
         <f aca="true">TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-05-20  10-59</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>324</v>
-      </c>
-      <c r="F2" s="3"/>
+        <v>2019-05-20  16-30</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>329</v>
+      </c>
+      <c r="F2" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Changed HH form and swahili translations (#17)
- Separated the Household registration Name field into First, Middle, and Last name.
- Replaced the word "family name" with "last name".
- Changed the relevancy of the child under 5 note which is now displayed only when either the exact dob or an estimated age is entered. Also, made sure that the note is not displayed if the dob or age is out of range.
- Added Samira's Swahili translation suggestions.
</commit_message>
<xml_diff>
--- a/forms/contact/clinic-create.xlsx
+++ b/forms/contact/clinic-create.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="349">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -179,16 +179,28 @@
     <t xml:space="preserve">${first_name_contact}</t>
   </si>
   <si>
-    <t xml:space="preserve">family_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Family name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jina la ukoo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${family_name_contact}</t>
+    <t xml:space="preserve">middle_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle name </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jina la baba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${middle_name_contact}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jina la babu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${last_name_contact}</t>
   </si>
   <si>
     <t xml:space="preserve">Full name</t>
@@ -317,7 +329,7 @@
     <t xml:space="preserve">SAY: For each person, I will ask some basic details about who they are, starting with either the head of household or best contact person for this household. Who should I list as the person I can reach out to coordinate care for themselves and other members of this household? This person should be reachable by phone.</t>
   </si>
   <si>
-    <t xml:space="preserve">SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mkuu wa kaya au mtu mzima yoyote ambaye naweza kuwasiliana naye kwenye nyumba hii. Je, ni nani atakayekuwa mtu ninayeweza  kukutana naye ili kuratibu utowaji wa huduma kwake mwenyewe na watu wengine walioko kwenye familia?  Mtu huyu awe anapatikana kupitia mawasiliano ya simu.</t>
+    <t xml:space="preserve">SEMA: Kwa kila mmoja, nitawauliza baadhi ya taarifa za msingi za utambulisho wenu, tukianza na mkuu wa kaya au mtu mzima yoyote ambaye naweza kuwasiliana naye kwenye nyumba hii. Je, ni nani anaweza kuratibu utowaji wa huduma kwenye familia hii?  Mtu huyu awe na simu kurahisisha mawasiliano.</t>
   </si>
   <si>
     <t xml:space="preserve">init</t>
@@ -338,7 +350,7 @@
     <t xml:space="preserve">ASK: What is the first name of the best contact person for your household?</t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: Ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu?</t>
+    <t xml:space="preserve">ULIZA: Ni lipi jina la kwanza la mtu ambaye naweza kuwasiliana naye kwenye kaya yenu? </t>
   </si>
   <si>
     <t xml:space="preserve">string-length(translate(.," ","")) &gt;= 2</t>
@@ -347,22 +359,43 @@
     <t xml:space="preserve">Enter a first name</t>
   </si>
   <si>
-    <t xml:space="preserve">family_name_contact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASK: What is their family name?</t>
+    <t xml:space="preserve">Jaza jina la mwanzo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">middle_name_contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASK: What is the middle name?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULIZA: Ni lipi jina la baba yake?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enter a middle name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaza jina  la baba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_name_contact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASK: What is their last name?</t>
   </si>
   <si>
     <t xml:space="preserve">ULIZA: Ni lipi jina la babu yake?</t>
   </si>
   <si>
-    <t xml:space="preserve">Enter a family name</t>
+    <t xml:space="preserve">Enter a last name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaza jina la babu</t>
   </si>
   <si>
     <t xml:space="preserve">name_contact</t>
   </si>
   <si>
-    <t xml:space="preserve">concat(${first_name_contact}," ",${family_name_contact})</t>
+    <t xml:space="preserve">concat(${first_name_contact}," ",${middle_name_contact}," ",${last_name_contact})</t>
   </si>
   <si>
     <t xml:space="preserve">select_one sex</t>
@@ -449,7 +482,7 @@
     <t xml:space="preserve">ASK: What is the best contact phone number for ${first_name_contact}?</t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: Je ni ipi nambari yake nzuri ya mawasilaano?</t>
+    <t xml:space="preserve">ULIZA: Je ni ipi nambari yake ya mawasiliano? </t>
   </si>
   <si>
     <t xml:space="preserve">regex(.,'^(\+255|0)[0-9]{9}$')</t>
@@ -467,7 +500,7 @@
     <t xml:space="preserve">ASK: Is there another phone number used by ${first_name_contact} or another member of the household?</t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: Je kuna nambari ya ziada anayotumia kuwasilaina?</t>
+    <t xml:space="preserve">ULIZA: Je kuna nambari ya ziada anayotumia kuwasiliana? </t>
   </si>
   <si>
     <t xml:space="preserve">You can leave this blank if there is only one good contact number for this household</t>
@@ -533,7 +566,19 @@
     <t xml:space="preserve">ULIZA: Ni lipi jina lake la kwanza? </t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: Ni lipi jina lake la babu? </t>
+    <t xml:space="preserve">Jaza jina la kwanza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASK: What is their middle name?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULIZA: Ni lipi jina la baba yake? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaza jina la baba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULIZA: Ni lipi jina la babu yake? </t>
   </si>
   <si>
     <t xml:space="preserve">first_name_c</t>
@@ -542,13 +587,19 @@
     <t xml:space="preserve">../first_name</t>
   </si>
   <si>
-    <t xml:space="preserve">family_name_c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">../family_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">concat(${first_name_c}," ",${family_name_c})</t>
+    <t xml:space="preserve">middle_name_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../middle_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_name_c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">../last_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">concat(${first_name_c}," ",${middle_name_c}," ",${last_name_c})</t>
   </si>
   <si>
     <t xml:space="preserve">Enter ${first_name_c}'s sex</t>
@@ -587,7 +638,7 @@
     <t xml:space="preserve">${exact_dob_known_c}="no"</t>
   </si>
   <si>
-    <t xml:space="preserve">. &gt; 5 and . &lt;= 100</t>
+    <t xml:space="preserve">. &gt;= 5 and . &lt;= 100</t>
   </si>
   <si>
     <t xml:space="preserve">Age must be between 5 and 100. For children under 5 years of age, a more exact birthdate must be captured.  Please select "Yes" to the prior question and do your best to capture more exact birthdate information about the child.</t>
@@ -599,7 +650,7 @@
     <t xml:space="preserve">yob</t>
   </si>
   <si>
-    <t xml:space="preserve">format-date-time(today(),"%Y")  - ../age_estimate</t>
+    <t xml:space="preserve">if(../age_estimate != '', format-date-time(today(),"%Y") - ../age_estimate, 1900)</t>
   </si>
   <si>
     <t xml:space="preserve">dob</t>
@@ -608,7 +659,7 @@
     <t xml:space="preserve">ASK: What is ${first_name_c}'s date of birth?</t>
   </si>
   <si>
-    <t xml:space="preserve">ULIZA: Ipi ni tarehe yake kuzaliwa</t>
+    <t xml:space="preserve">ULIZA: Ni ipi tarehe yake ya kuzaliwa? </t>
   </si>
   <si>
     <t xml:space="preserve">${exact_dob_known_c}="yes"</t>
@@ -620,7 +671,7 @@
     <t xml:space="preserve">You've entered a birthdate either in the future or very long ago - confirm that you've entered it properly.</t>
   </si>
   <si>
-    <t xml:space="preserve">Je umeingiza umri sahihi- hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya Zaidi ya miaka 5 nyuma.</t>
+    <t xml:space="preserve">Je umeingiza umri sahihi? Hakikisha umeingiza kwa usahihi. Kwa watoto walio chini ya miaka 5, hakikisha kuwa tarehe yao si ya zaidi ya miaka 5 nyuma.</t>
   </si>
   <si>
     <t xml:space="preserve">format-date(if(../dob != '', ../dob,concat(../yob, '-01-01')), '%Y-%m-%d')</t>
@@ -632,6 +683,12 @@
     <t xml:space="preserve">../date_of_birth</t>
   </si>
   <si>
+    <t xml:space="preserve">is_exact_dob_in_range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if((../date_of_birth_c &lt;= date-time(decimal-date-time(today())) and ../date_of_birth_c &gt;= date-time(decimal-date-time(today() - (100 * 365.25)))),1,0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">reproductive_age</t>
   </si>
   <si>
@@ -650,10 +707,10 @@
     <t xml:space="preserve">SAY: From this registration, I've seen that you have a child under 5 who can benefit from this national program. Therefore, I'm asking for your permission to come back and check up on all issues related to their health care, nutrition, and child development. I would be grateful for your permission.</t>
   </si>
   <si>
-    <t xml:space="preserve">SEMA kutokanana usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe, na maendeleo yao. Nitafurahi kama nitapata ridhaa yenu.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">${is_under_5_binary}=1</t>
+    <t xml:space="preserve">SEMA: Kutokana na usajili huu nimeona kuna watoto walio chini ya umri wa miaka 5 ambao wanaweza kunufaika na mradi huu wa kitaifa. Kwahivyo naomba ridhaa ya kurudi tena ili nije kuangalia maswala yote yanayohusiana na huduma zao za afya, lishe, na maendeleo yao. Nitafurahi kama nitapata ridhaa yenu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${exact_dob_known_c}="yes" and    ${is_under_5_binary}=1 and  ${is_exact_dob_in_range} = 1</t>
   </si>
   <si>
     <t xml:space="preserve">return_women_note</t>
@@ -701,7 +758,7 @@
     <t xml:space="preserve">_The purpose of the following questions regarding the household location is to help you locate this house again when it is time to return for another visit to the people who live here. Enter the information that you will need to help you easily find this house again when you need to before you approach the household. What is the address of this household?_</t>
   </si>
   <si>
-    <t xml:space="preserve">Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudia kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kuirudia tena. Ni ipi anuani ya nyumba hii?</t>
+    <t xml:space="preserve">Lengo la maswali haya yanayouliza kuhusu eneo la kaya ni kwajili ya kukusaidia kuweza kuitambua kwa urahisi kaya wakati wa kutaka kurudi kufanya matembeleo mengine kwa watu wanaoishi humu. Ingiza taarifa zitazoweza kukusaidia kiurahisi kuitambua kaya hii pindi unapotaka kurudi tena. Ni ipi anuani ya nyumba hii?</t>
   </si>
   <si>
     <t xml:space="preserve">kitongoji</t>
@@ -803,7 +860,7 @@
     <t xml:space="preserve">clinic</t>
   </si>
   <si>
-    <t xml:space="preserve">concat('Nyumba ya ' , ../../contact/first_name,../../contact/last_name, '  - Nyumba no. ',../../household_location/house_number)</t>
+    <t xml:space="preserve">concat('Nyumba ya ' , ../../contact/first_name, '  - Nyumba no. ',../../household_location/house_number)</t>
   </si>
   <si>
     <t xml:space="preserve">geolocation</t>
@@ -1030,7 +1087,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1058,6 +1115,12 @@
       <name val="Sans"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Sans"/>
+      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -1126,10 +1189,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1142,7 +1201,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1163,7 +1226,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q1048576"/>
+  <dimension ref="A1:Q114"/>
   <sheetFormatPr defaultRowHeight="13" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.7"/>
@@ -1475,16 +1538,16 @@
         <v>30</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>1</v>
+        <v>53</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="L20" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1492,7 +1555,7 @@
         <v>30</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>57</v>
@@ -1514,8 +1577,11 @@
       <c r="C22" s="1" t="s">
         <v>61</v>
       </c>
+      <c r="D22" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="L22" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1523,12 +1589,9 @@
         <v>30</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D23" s="1" t="s">
         <v>65</v>
       </c>
       <c r="L23" s="1" t="s">
@@ -1569,26 +1632,32 @@
         <v>74</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>75</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>19</v>
+        <v>76</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="L27" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1596,10 +1665,10 @@
         <v>30</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1607,113 +1676,107 @@
         <v>30</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>84</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>83</v>
+        <v>17</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I33" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="J33" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="N33" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="O33" s="1" t="s">
-        <v>91</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="J34" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="N34" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="O34" s="1" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>96</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>82</v>
+        <v>97</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>99</v>
+        <v>17</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>100</v>
@@ -1724,132 +1787,136 @@
       <c r="D37" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E37" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>104</v>
+      <c r="G37" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>47</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="J38" s="1" t="s">
         <v>108</v>
       </c>
+      <c r="K38" s="1" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="L39" s="1" t="s">
         <v>110</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J39" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>47</v>
       </c>
+      <c r="I40" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>115</v>
+        <v>30</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>47</v>
+        <v>120</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>123</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F42" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>30</v>
+        <v>126</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="J43" s="0"/>
-      <c r="K43" s="0"/>
-      <c r="L43" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>129</v>
+        <v>87</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>130</v>
@@ -1878,79 +1945,102 @@
     </row>
     <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="C45" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="D45" s="1" t="s">
+      <c r="J45" s="0"/>
+      <c r="K45" s="0"/>
+      <c r="L45" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I45" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="J45" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="B46" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="D46" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="E46" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F46" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D46" s="1" t="s">
+      <c r="I46" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I46" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="J46" s="1" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="N46" s="1" t="s">
-        <v>146</v>
-      </c>
-      <c r="O46" s="1" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="L47" s="1" t="s">
+      <c r="C47" s="1" t="s">
         <v>149</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="J47" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="L48" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="I48" s="1" t="s">
         <v>151</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K48" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="N48" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="O48" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1958,199 +2048,214 @@
         <v>30</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>96</v>
+        <v>161</v>
+      </c>
+      <c r="L50" s="1" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>155</v>
+        <v>163</v>
+      </c>
+      <c r="L51" s="1" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>156</v>
+        <v>29</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G52" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q52" s="1" t="s">
-        <v>160</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>92</v>
+        <v>17</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>163</v>
+        <v>19</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>21</v>
+        <v>167</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>19</v>
+        <v>169</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>170</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P54" s="1" t="s">
-        <v>164</v>
+        <v>40</v>
+      </c>
+      <c r="Q54" s="1" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>41</v>
+        <v>172</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="L55" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="P55" s="1" t="s">
-        <v>43</v>
+        <v>173</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J56" s="1" t="s">
-        <v>104</v>
+        <v>19</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P56" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>99</v>
+        <v>21</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>108</v>
+        <v>19</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="P57" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>169</v>
+        <v>44</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="L59" s="1" t="s">
-        <v>171</v>
+        <v>49</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K59" s="1" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="L60" s="1" t="s">
-        <v>172</v>
+        <v>53</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>47</v>
+        <v>183</v>
+      </c>
+      <c r="L61" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2158,27 +2263,21 @@
         <v>30</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>115</v>
+        <v>30</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>47</v>
+        <v>187</v>
+      </c>
+      <c r="L63" s="1" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2186,91 +2285,63 @@
         <v>30</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>179</v>
+        <v>1</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>181</v>
+        <v>122</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F65" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="L65" s="0"/>
     </row>
     <row r="66" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L66" s="3" t="s">
-        <v>189</v>
+      <c r="B66" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="L66" s="1" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>190</v>
+        <v>64</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F67" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>196</v>
-      </c>
     </row>
     <row r="68" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>63</v>
+        <v>196</v>
       </c>
       <c r="L68" s="1" t="s">
         <v>197</v>
@@ -2278,424 +2349,446 @@
     </row>
     <row r="69" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="L69" s="1" t="s">
+      <c r="C69" s="1" t="s">
         <v>199</v>
       </c>
+      <c r="D69" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K69" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="L69" s="0"/>
     </row>
     <row r="70" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="L70" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="L71" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>207</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="C72" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>67</v>
+      </c>
+      <c r="L72" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="G73" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="L73" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="L74" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="L75" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="L76" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G78" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="G74" s="1" t="s">
+    <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="G79" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="1" t="s">
+    <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B75" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C75" s="1" t="s">
+      <c r="B80" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="L76" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L77" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B78" s="1" t="s">
+    <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B81" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="L78" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>154</v>
+      <c r="L81" s="1" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>40</v>
+        <v>82</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>40</v>
+        <v>84</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="E84" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I84" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="J84" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="K84" s="1" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>99</v>
+        <v>236</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>229</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="E85" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I85" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="J85" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="K85" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="N85" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="O85" s="1" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="E86" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I86" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="J86" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="K86" s="1" t="s">
-        <v>241</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
-        <v>242</v>
+        <v>17</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>47</v>
+        <v>239</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="E88" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F88" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="I88" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="J88" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="K88" s="1" t="s">
-        <v>252</v>
+        <v>242</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="J90" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="N90" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="O90" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="J93" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L92" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="P92" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L93" s="1" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1" t="s">
-        <v>30</v>
-      </c>
       <c r="B94" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="L94" s="1" t="s">
-        <v>260</v>
+        <v>237</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>30</v>
+        <v>96</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>39</v>
+        <v>272</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L95" s="1" t="s">
-        <v>261</v>
+        <v>273</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>274</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="L96" s="1" t="s">
-        <v>264</v>
+        <v>19</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2703,13 +2796,16 @@
         <v>30</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>265</v>
+        <v>41</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>266</v>
+        <v>19</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>267</v>
+        <v>42</v>
+      </c>
+      <c r="P97" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2717,13 +2813,13 @@
         <v>30</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>224</v>
+        <v>1</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>268</v>
+        <v>19</v>
       </c>
       <c r="L98" s="1" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2731,13 +2827,13 @@
         <v>30</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>229</v>
+        <v>277</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="L99" s="1" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2745,13 +2841,13 @@
         <v>30</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>236</v>
+        <v>39</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
       <c r="L100" s="1" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2759,13 +2855,13 @@
         <v>30</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="L101" s="1" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2773,13 +2869,13 @@
         <v>30</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="L102" s="1" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2787,76 +2883,145 @@
         <v>30</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>279</v>
+        <v>243</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="L103" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="L104" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="L105" s="1" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="L106" s="1" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="L107" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="L108" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B104" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C104" s="1" t="s">
+      <c r="B109" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C109" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="L105" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L106" s="1" t="s">
+    <row r="110" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="L110" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L111" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L112" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B113" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="L107" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="108" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="1" t="s">
+    <row r="114" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B108" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="109" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B109" s="1" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="B114" s="1" t="s">
+        <v>275</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="1" right="1" top="1.66666666666667" bottom="1.66666666666667" header="1" footer="1"/>
@@ -2885,7 +3050,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -2899,198 +3064,198 @@
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>307</v>
+        <v>326</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>
@@ -3123,40 +3288,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="C2" s="6" t="str">
         <f aca="true">TEXT(NOW(),"yyyy-mm-dd_HH-MM")</f>
-        <v>2019-05-20  16-30</v>
+        <v>2019-05-22  16-08</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="F2" s="5"/>
     </row>

</xml_diff>